<commit_message>
260830 add harris, elabe and ifop polls
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30EA786-2735-B940-949E-4FF447D0D908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7768A5-60B2-7345-BDEC-765E6E48F094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="6700" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="40">
   <si>
     <t>id</t>
   </si>
@@ -538,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AB64"/>
+  <dimension ref="A1:AB75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -5313,6 +5313,808 @@
         <v>0</v>
       </c>
     </row>
+    <row r="65" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>17</v>
+      </c>
+      <c r="B65">
+        <v>2026</v>
+      </c>
+      <c r="C65">
+        <v>8</v>
+      </c>
+      <c r="D65">
+        <v>18</v>
+      </c>
+      <c r="E65">
+        <v>8</v>
+      </c>
+      <c r="F65">
+        <v>19</v>
+      </c>
+      <c r="G65" t="s">
+        <v>31</v>
+      </c>
+      <c r="H65" t="s">
+        <v>32</v>
+      </c>
+      <c r="I65" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65">
+        <v>1482</v>
+      </c>
+      <c r="K65">
+        <v>0</v>
+      </c>
+      <c r="L65">
+        <v>1</v>
+      </c>
+      <c r="M65">
+        <v>1</v>
+      </c>
+      <c r="N65">
+        <v>1</v>
+      </c>
+      <c r="O65">
+        <v>17</v>
+      </c>
+      <c r="P65">
+        <v>3</v>
+      </c>
+      <c r="Q65">
+        <v>10</v>
+      </c>
+      <c r="S65">
+        <v>3</v>
+      </c>
+      <c r="T65">
+        <v>17</v>
+      </c>
+      <c r="V65">
+        <v>7</v>
+      </c>
+      <c r="X65">
+        <v>3</v>
+      </c>
+      <c r="Z65">
+        <v>35</v>
+      </c>
+      <c r="AA65">
+        <v>4</v>
+      </c>
+      <c r="AB65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>17</v>
+      </c>
+      <c r="B66">
+        <v>2026</v>
+      </c>
+      <c r="C66">
+        <v>8</v>
+      </c>
+      <c r="D66">
+        <v>18</v>
+      </c>
+      <c r="E66">
+        <v>8</v>
+      </c>
+      <c r="F66">
+        <v>19</v>
+      </c>
+      <c r="G66" t="s">
+        <v>31</v>
+      </c>
+      <c r="H66" t="s">
+        <v>32</v>
+      </c>
+      <c r="I66" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66">
+        <v>1482</v>
+      </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
+      <c r="L66">
+        <v>1</v>
+      </c>
+      <c r="M66">
+        <v>1</v>
+      </c>
+      <c r="N66">
+        <v>1</v>
+      </c>
+      <c r="O66">
+        <v>17</v>
+      </c>
+      <c r="P66">
+        <v>2</v>
+      </c>
+      <c r="Q66">
+        <v>11</v>
+      </c>
+      <c r="S66">
+        <v>3</v>
+      </c>
+      <c r="U66">
+        <v>15</v>
+      </c>
+      <c r="V66">
+        <v>9</v>
+      </c>
+      <c r="X66">
+        <v>2</v>
+      </c>
+      <c r="Z66">
+        <v>37</v>
+      </c>
+      <c r="AA66">
+        <v>3</v>
+      </c>
+      <c r="AB66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>17</v>
+      </c>
+      <c r="B67">
+        <v>2026</v>
+      </c>
+      <c r="C67">
+        <v>8</v>
+      </c>
+      <c r="D67">
+        <v>18</v>
+      </c>
+      <c r="E67">
+        <v>8</v>
+      </c>
+      <c r="F67">
+        <v>19</v>
+      </c>
+      <c r="G67" t="s">
+        <v>31</v>
+      </c>
+      <c r="H67" t="s">
+        <v>32</v>
+      </c>
+      <c r="I67" t="s">
+        <v>12</v>
+      </c>
+      <c r="J67">
+        <v>1482</v>
+      </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
+      <c r="L67">
+        <v>1</v>
+      </c>
+      <c r="M67">
+        <v>1</v>
+      </c>
+      <c r="N67">
+        <v>1</v>
+      </c>
+      <c r="O67">
+        <v>17</v>
+      </c>
+      <c r="P67">
+        <v>3</v>
+      </c>
+      <c r="R67">
+        <v>8</v>
+      </c>
+      <c r="S67">
+        <v>4</v>
+      </c>
+      <c r="T67">
+        <v>19</v>
+      </c>
+      <c r="V67">
+        <v>7</v>
+      </c>
+      <c r="X67">
+        <v>2</v>
+      </c>
+      <c r="Z67">
+        <v>35</v>
+      </c>
+      <c r="AA67">
+        <v>4</v>
+      </c>
+      <c r="AB67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>17</v>
+      </c>
+      <c r="B68">
+        <v>2026</v>
+      </c>
+      <c r="C68">
+        <v>8</v>
+      </c>
+      <c r="D68">
+        <v>18</v>
+      </c>
+      <c r="E68">
+        <v>8</v>
+      </c>
+      <c r="F68">
+        <v>19</v>
+      </c>
+      <c r="G68" t="s">
+        <v>31</v>
+      </c>
+      <c r="H68" t="s">
+        <v>32</v>
+      </c>
+      <c r="I68" t="s">
+        <v>12</v>
+      </c>
+      <c r="J68">
+        <v>1464</v>
+      </c>
+      <c r="K68">
+        <v>0</v>
+      </c>
+      <c r="L68">
+        <v>1</v>
+      </c>
+      <c r="M68">
+        <v>1</v>
+      </c>
+      <c r="N68">
+        <v>1</v>
+      </c>
+      <c r="O68">
+        <v>17</v>
+      </c>
+      <c r="P68">
+        <v>3</v>
+      </c>
+      <c r="R68">
+        <v>8</v>
+      </c>
+      <c r="S68">
+        <v>4</v>
+      </c>
+      <c r="U68">
+        <v>14</v>
+      </c>
+      <c r="V68">
+        <v>9</v>
+      </c>
+      <c r="X68">
+        <v>2</v>
+      </c>
+      <c r="Z68">
+        <v>38</v>
+      </c>
+      <c r="AA68">
+        <v>4</v>
+      </c>
+      <c r="AB68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>18</v>
+      </c>
+      <c r="B69">
+        <v>2026</v>
+      </c>
+      <c r="C69">
+        <v>8</v>
+      </c>
+      <c r="D69">
+        <v>24</v>
+      </c>
+      <c r="E69">
+        <v>8</v>
+      </c>
+      <c r="F69">
+        <v>25</v>
+      </c>
+      <c r="G69" t="s">
+        <v>11</v>
+      </c>
+      <c r="H69" t="s">
+        <v>13</v>
+      </c>
+      <c r="I69" t="s">
+        <v>12</v>
+      </c>
+      <c r="J69">
+        <v>920</v>
+      </c>
+      <c r="K69">
+        <v>0</v>
+      </c>
+      <c r="L69">
+        <v>1</v>
+      </c>
+      <c r="M69">
+        <v>0.5</v>
+      </c>
+      <c r="N69">
+        <v>1</v>
+      </c>
+      <c r="O69">
+        <v>17</v>
+      </c>
+      <c r="P69">
+        <v>3</v>
+      </c>
+      <c r="Q69">
+        <v>12</v>
+      </c>
+      <c r="S69">
+        <v>3</v>
+      </c>
+      <c r="T69">
+        <v>18</v>
+      </c>
+      <c r="V69">
+        <v>8</v>
+      </c>
+      <c r="X69">
+        <v>1.5</v>
+      </c>
+      <c r="Z69">
+        <v>33</v>
+      </c>
+      <c r="AA69">
+        <v>3.5</v>
+      </c>
+      <c r="AB69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>18</v>
+      </c>
+      <c r="B70">
+        <v>2026</v>
+      </c>
+      <c r="C70">
+        <v>8</v>
+      </c>
+      <c r="D70">
+        <v>24</v>
+      </c>
+      <c r="E70">
+        <v>8</v>
+      </c>
+      <c r="F70">
+        <v>25</v>
+      </c>
+      <c r="G70" t="s">
+        <v>11</v>
+      </c>
+      <c r="H70" t="s">
+        <v>13</v>
+      </c>
+      <c r="I70" t="s">
+        <v>12</v>
+      </c>
+      <c r="J70">
+        <v>909</v>
+      </c>
+      <c r="K70">
+        <v>0</v>
+      </c>
+      <c r="L70">
+        <v>1</v>
+      </c>
+      <c r="M70">
+        <v>0.5</v>
+      </c>
+      <c r="N70">
+        <v>0.5</v>
+      </c>
+      <c r="O70">
+        <v>17</v>
+      </c>
+      <c r="P70">
+        <v>3</v>
+      </c>
+      <c r="Q70">
+        <v>15</v>
+      </c>
+      <c r="S70">
+        <v>3</v>
+      </c>
+      <c r="U70">
+        <v>14</v>
+      </c>
+      <c r="V70">
+        <v>9</v>
+      </c>
+      <c r="X70">
+        <v>1.5</v>
+      </c>
+      <c r="Z70">
+        <v>34</v>
+      </c>
+      <c r="AA70">
+        <v>3</v>
+      </c>
+      <c r="AB70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>18</v>
+      </c>
+      <c r="B71">
+        <v>2026</v>
+      </c>
+      <c r="C71">
+        <v>8</v>
+      </c>
+      <c r="D71">
+        <v>24</v>
+      </c>
+      <c r="E71">
+        <v>8</v>
+      </c>
+      <c r="F71">
+        <v>25</v>
+      </c>
+      <c r="G71" t="s">
+        <v>11</v>
+      </c>
+      <c r="H71" t="s">
+        <v>13</v>
+      </c>
+      <c r="I71" t="s">
+        <v>12</v>
+      </c>
+      <c r="J71">
+        <v>925</v>
+      </c>
+      <c r="K71">
+        <v>0</v>
+      </c>
+      <c r="L71">
+        <v>1</v>
+      </c>
+      <c r="M71">
+        <v>0.5</v>
+      </c>
+      <c r="N71">
+        <v>1</v>
+      </c>
+      <c r="O71">
+        <v>18</v>
+      </c>
+      <c r="Q71">
+        <v>15</v>
+      </c>
+      <c r="T71">
+        <v>19</v>
+      </c>
+      <c r="V71">
+        <v>8</v>
+      </c>
+      <c r="X71">
+        <v>2.5</v>
+      </c>
+      <c r="Z71">
+        <v>33</v>
+      </c>
+      <c r="AA71">
+        <v>3.5</v>
+      </c>
+      <c r="AB71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>18</v>
+      </c>
+      <c r="B72">
+        <v>2026</v>
+      </c>
+      <c r="C72">
+        <v>8</v>
+      </c>
+      <c r="D72">
+        <v>24</v>
+      </c>
+      <c r="E72">
+        <v>8</v>
+      </c>
+      <c r="F72">
+        <v>25</v>
+      </c>
+      <c r="G72" t="s">
+        <v>11</v>
+      </c>
+      <c r="H72" t="s">
+        <v>13</v>
+      </c>
+      <c r="I72" t="s">
+        <v>12</v>
+      </c>
+      <c r="J72">
+        <v>898</v>
+      </c>
+      <c r="K72">
+        <v>0</v>
+      </c>
+      <c r="L72">
+        <v>1</v>
+      </c>
+      <c r="M72">
+        <v>0.5</v>
+      </c>
+      <c r="N72">
+        <v>1.5</v>
+      </c>
+      <c r="O72">
+        <v>18.5</v>
+      </c>
+      <c r="Q72">
+        <v>17</v>
+      </c>
+      <c r="U72">
+        <v>15</v>
+      </c>
+      <c r="V72">
+        <v>9</v>
+      </c>
+      <c r="X72">
+        <v>2</v>
+      </c>
+      <c r="Z72">
+        <v>34</v>
+      </c>
+      <c r="AA72">
+        <v>3</v>
+      </c>
+      <c r="AB72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>18</v>
+      </c>
+      <c r="B73">
+        <v>2026</v>
+      </c>
+      <c r="C73">
+        <v>8</v>
+      </c>
+      <c r="D73">
+        <v>24</v>
+      </c>
+      <c r="E73">
+        <v>8</v>
+      </c>
+      <c r="F73">
+        <v>25</v>
+      </c>
+      <c r="G73" t="s">
+        <v>11</v>
+      </c>
+      <c r="H73" t="s">
+        <v>13</v>
+      </c>
+      <c r="I73" t="s">
+        <v>12</v>
+      </c>
+      <c r="J73">
+        <v>889</v>
+      </c>
+      <c r="K73">
+        <v>0</v>
+      </c>
+      <c r="L73">
+        <v>1</v>
+      </c>
+      <c r="M73">
+        <v>0.5</v>
+      </c>
+      <c r="N73">
+        <v>1.5</v>
+      </c>
+      <c r="O73">
+        <v>19</v>
+      </c>
+      <c r="R73">
+        <v>12</v>
+      </c>
+      <c r="T73">
+        <v>21</v>
+      </c>
+      <c r="V73">
+        <v>8</v>
+      </c>
+      <c r="X73">
+        <v>2</v>
+      </c>
+      <c r="Z73">
+        <v>34</v>
+      </c>
+      <c r="AA73">
+        <v>2.5</v>
+      </c>
+      <c r="AB73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>19</v>
+      </c>
+      <c r="B74">
+        <v>2026</v>
+      </c>
+      <c r="C74">
+        <v>8</v>
+      </c>
+      <c r="D74">
+        <v>26</v>
+      </c>
+      <c r="E74">
+        <v>8</v>
+      </c>
+      <c r="F74">
+        <v>28</v>
+      </c>
+      <c r="G74" t="s">
+        <v>29</v>
+      </c>
+      <c r="H74" t="s">
+        <v>28</v>
+      </c>
+      <c r="I74" t="s">
+        <v>12</v>
+      </c>
+      <c r="J74">
+        <v>1000</v>
+      </c>
+      <c r="K74">
+        <v>1</v>
+      </c>
+      <c r="L74">
+        <v>1</v>
+      </c>
+      <c r="M74">
+        <v>0.5</v>
+      </c>
+      <c r="N74">
+        <v>1.5</v>
+      </c>
+      <c r="O74">
+        <v>14</v>
+      </c>
+      <c r="P74">
+        <v>3</v>
+      </c>
+      <c r="Q74">
+        <v>11.5</v>
+      </c>
+      <c r="S74">
+        <v>3.5</v>
+      </c>
+      <c r="T74">
+        <v>17</v>
+      </c>
+      <c r="V74">
+        <v>6.5</v>
+      </c>
+      <c r="W74">
+        <v>2</v>
+      </c>
+      <c r="X74">
+        <v>3</v>
+      </c>
+      <c r="Z74">
+        <v>34</v>
+      </c>
+      <c r="AA74">
+        <v>4</v>
+      </c>
+      <c r="AB74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>19</v>
+      </c>
+      <c r="B75">
+        <v>2026</v>
+      </c>
+      <c r="C75">
+        <v>8</v>
+      </c>
+      <c r="D75">
+        <v>26</v>
+      </c>
+      <c r="E75">
+        <v>8</v>
+      </c>
+      <c r="F75">
+        <v>28</v>
+      </c>
+      <c r="G75" t="s">
+        <v>29</v>
+      </c>
+      <c r="H75" t="s">
+        <v>28</v>
+      </c>
+      <c r="I75" t="s">
+        <v>12</v>
+      </c>
+      <c r="J75">
+        <v>1000</v>
+      </c>
+      <c r="K75">
+        <v>1</v>
+      </c>
+      <c r="L75">
+        <v>1</v>
+      </c>
+      <c r="M75">
+        <v>0.5</v>
+      </c>
+      <c r="N75">
+        <v>1.5</v>
+      </c>
+      <c r="O75">
+        <v>14</v>
+      </c>
+      <c r="P75">
+        <v>3</v>
+      </c>
+      <c r="Q75">
+        <v>14</v>
+      </c>
+      <c r="S75">
+        <v>3</v>
+      </c>
+      <c r="U75">
+        <v>12</v>
+      </c>
+      <c r="V75">
+        <v>9.5</v>
+      </c>
+      <c r="W75">
+        <v>2.5</v>
+      </c>
+      <c r="X75">
+        <v>2</v>
+      </c>
+      <c r="Z75">
+        <v>34.5</v>
+      </c>
+      <c r="AA75">
+        <v>4</v>
+      </c>
+      <c r="AB75">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update data until sept 2
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7768A5-60B2-7345-BDEC-765E6E48F094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF229AB-8246-E246-BDEE-540E7AF3F4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="6700" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="41">
   <si>
     <t>id</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>verian</t>
+  </si>
+  <si>
+    <t>cluster17</t>
   </si>
 </sst>
 </file>
@@ -536,9 +539,29 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6649D996-6833-C548-BBDE-C83189B87AE7}">
+  <we:reference id="93533c7f-4dc5-468f-aba4-1c008e1a7ac8" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200003101" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AB75"/>
+  <dimension ref="A1:AB83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -6115,6 +6138,604 @@
         <v>0</v>
       </c>
     </row>
+    <row r="76" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>20</v>
+      </c>
+      <c r="B76">
+        <v>2026</v>
+      </c>
+      <c r="C76">
+        <v>7</v>
+      </c>
+      <c r="D76">
+        <v>22</v>
+      </c>
+      <c r="E76">
+        <v>7</v>
+      </c>
+      <c r="F76">
+        <v>24</v>
+      </c>
+      <c r="G76" t="s">
+        <v>40</v>
+      </c>
+      <c r="H76" t="s">
+        <v>32</v>
+      </c>
+      <c r="I76" t="s">
+        <v>12</v>
+      </c>
+      <c r="J76">
+        <v>1207</v>
+      </c>
+      <c r="K76">
+        <v>0</v>
+      </c>
+      <c r="L76">
+        <v>1</v>
+      </c>
+      <c r="M76">
+        <v>0.1</v>
+      </c>
+      <c r="N76">
+        <v>0.9</v>
+      </c>
+      <c r="O76">
+        <v>18.2</v>
+      </c>
+      <c r="P76">
+        <v>2</v>
+      </c>
+      <c r="Q76">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="S76">
+        <v>2.8</v>
+      </c>
+      <c r="T76">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="V76">
+        <v>7.8</v>
+      </c>
+      <c r="W76">
+        <v>2.9</v>
+      </c>
+      <c r="X76">
+        <v>3.2</v>
+      </c>
+      <c r="Z76">
+        <v>30.1</v>
+      </c>
+      <c r="AA76">
+        <v>3.8</v>
+      </c>
+      <c r="AB76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>20</v>
+      </c>
+      <c r="B77">
+        <v>2026</v>
+      </c>
+      <c r="C77">
+        <v>7</v>
+      </c>
+      <c r="D77">
+        <v>22</v>
+      </c>
+      <c r="E77">
+        <v>7</v>
+      </c>
+      <c r="F77">
+        <v>24</v>
+      </c>
+      <c r="G77" t="s">
+        <v>40</v>
+      </c>
+      <c r="H77" t="s">
+        <v>32</v>
+      </c>
+      <c r="I77" t="s">
+        <v>12</v>
+      </c>
+      <c r="J77">
+        <v>1209</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+      <c r="L77">
+        <v>1</v>
+      </c>
+      <c r="M77">
+        <v>0.1</v>
+      </c>
+      <c r="N77">
+        <v>1</v>
+      </c>
+      <c r="O77">
+        <v>18.3</v>
+      </c>
+      <c r="P77">
+        <v>1.8</v>
+      </c>
+      <c r="Q77">
+        <v>10.3</v>
+      </c>
+      <c r="S77">
+        <v>3.1</v>
+      </c>
+      <c r="U77">
+        <v>13.8</v>
+      </c>
+      <c r="V77">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="W77">
+        <v>3.9</v>
+      </c>
+      <c r="X77">
+        <v>4</v>
+      </c>
+      <c r="Z77">
+        <v>29.9</v>
+      </c>
+      <c r="AA77">
+        <v>4.2</v>
+      </c>
+      <c r="AB77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>21</v>
+      </c>
+      <c r="B78">
+        <v>2026</v>
+      </c>
+      <c r="C78">
+        <v>8</v>
+      </c>
+      <c r="D78">
+        <v>31</v>
+      </c>
+      <c r="E78">
+        <v>9</v>
+      </c>
+      <c r="F78">
+        <v>2</v>
+      </c>
+      <c r="G78" t="s">
+        <v>33</v>
+      </c>
+      <c r="H78" t="s">
+        <v>13</v>
+      </c>
+      <c r="I78" t="s">
+        <v>12</v>
+      </c>
+      <c r="J78">
+        <v>915</v>
+      </c>
+      <c r="K78">
+        <v>0</v>
+      </c>
+      <c r="L78">
+        <v>1</v>
+      </c>
+      <c r="M78">
+        <v>0.5</v>
+      </c>
+      <c r="N78">
+        <v>0.5</v>
+      </c>
+      <c r="O78">
+        <v>15</v>
+      </c>
+      <c r="P78">
+        <v>2.5</v>
+      </c>
+      <c r="Q78">
+        <v>12</v>
+      </c>
+      <c r="S78">
+        <v>4</v>
+      </c>
+      <c r="T78">
+        <v>19</v>
+      </c>
+      <c r="V78">
+        <v>7.5</v>
+      </c>
+      <c r="X78">
+        <v>2</v>
+      </c>
+      <c r="Z78">
+        <v>34.5</v>
+      </c>
+      <c r="AA78">
+        <v>3</v>
+      </c>
+      <c r="AB78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>21</v>
+      </c>
+      <c r="B79">
+        <v>2026</v>
+      </c>
+      <c r="C79">
+        <v>8</v>
+      </c>
+      <c r="D79">
+        <v>31</v>
+      </c>
+      <c r="E79">
+        <v>9</v>
+      </c>
+      <c r="F79">
+        <v>2</v>
+      </c>
+      <c r="G79" t="s">
+        <v>33</v>
+      </c>
+      <c r="H79" t="s">
+        <v>13</v>
+      </c>
+      <c r="I79" t="s">
+        <v>12</v>
+      </c>
+      <c r="J79">
+        <v>909</v>
+      </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
+      <c r="L79">
+        <v>1</v>
+      </c>
+      <c r="M79">
+        <v>0.5</v>
+      </c>
+      <c r="N79">
+        <v>0.5</v>
+      </c>
+      <c r="O79">
+        <v>15</v>
+      </c>
+      <c r="P79">
+        <v>2.5</v>
+      </c>
+      <c r="Q79">
+        <v>14</v>
+      </c>
+      <c r="S79">
+        <v>4</v>
+      </c>
+      <c r="U79">
+        <v>14</v>
+      </c>
+      <c r="V79">
+        <v>9.5</v>
+      </c>
+      <c r="X79">
+        <v>2.5</v>
+      </c>
+      <c r="Z79">
+        <v>35</v>
+      </c>
+      <c r="AA79">
+        <v>3</v>
+      </c>
+      <c r="AB79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>22</v>
+      </c>
+      <c r="B80">
+        <v>2026</v>
+      </c>
+      <c r="C80">
+        <v>8</v>
+      </c>
+      <c r="D80">
+        <v>31</v>
+      </c>
+      <c r="E80">
+        <v>9</v>
+      </c>
+      <c r="F80">
+        <v>1</v>
+      </c>
+      <c r="G80" t="s">
+        <v>40</v>
+      </c>
+      <c r="H80" t="s">
+        <v>32</v>
+      </c>
+      <c r="I80" t="s">
+        <v>12</v>
+      </c>
+      <c r="J80">
+        <v>1459</v>
+      </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
+      <c r="L80">
+        <v>1</v>
+      </c>
+      <c r="M80">
+        <v>0.1</v>
+      </c>
+      <c r="N80">
+        <v>0.9</v>
+      </c>
+      <c r="O80">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="P80">
+        <v>2.1</v>
+      </c>
+      <c r="Q80">
+        <v>11.6</v>
+      </c>
+      <c r="S80">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="T80">
+        <v>18.2</v>
+      </c>
+      <c r="V80">
+        <v>7.5</v>
+      </c>
+      <c r="W80">
+        <v>3.2</v>
+      </c>
+      <c r="X80">
+        <v>2.9</v>
+      </c>
+      <c r="Z80">
+        <v>30</v>
+      </c>
+      <c r="AA80">
+        <v>3.5</v>
+      </c>
+      <c r="AB80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>22</v>
+      </c>
+      <c r="B81">
+        <v>2026</v>
+      </c>
+      <c r="C81">
+        <v>8</v>
+      </c>
+      <c r="D81">
+        <v>31</v>
+      </c>
+      <c r="E81">
+        <v>9</v>
+      </c>
+      <c r="F81">
+        <v>1</v>
+      </c>
+      <c r="G81" t="s">
+        <v>40</v>
+      </c>
+      <c r="H81" t="s">
+        <v>32</v>
+      </c>
+      <c r="I81" t="s">
+        <v>12</v>
+      </c>
+      <c r="J81">
+        <v>1451</v>
+      </c>
+      <c r="K81">
+        <v>0</v>
+      </c>
+      <c r="L81">
+        <v>1</v>
+      </c>
+      <c r="M81">
+        <v>0.1</v>
+      </c>
+      <c r="N81">
+        <v>0.9</v>
+      </c>
+      <c r="O81">
+        <v>18.2</v>
+      </c>
+      <c r="P81">
+        <v>2.1</v>
+      </c>
+      <c r="Q81">
+        <v>11.5</v>
+      </c>
+      <c r="S81">
+        <v>2.5</v>
+      </c>
+      <c r="U81">
+        <v>13.5</v>
+      </c>
+      <c r="V81">
+        <v>8.9</v>
+      </c>
+      <c r="W81">
+        <v>4</v>
+      </c>
+      <c r="X81">
+        <v>2.8</v>
+      </c>
+      <c r="Z81">
+        <v>31.6</v>
+      </c>
+      <c r="AA81">
+        <v>4</v>
+      </c>
+      <c r="AB81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>23</v>
+      </c>
+      <c r="B82">
+        <v>2026</v>
+      </c>
+      <c r="C82">
+        <v>9</v>
+      </c>
+      <c r="D82">
+        <v>2</v>
+      </c>
+      <c r="E82">
+        <v>9</v>
+      </c>
+      <c r="F82">
+        <v>3</v>
+      </c>
+      <c r="G82" t="s">
+        <v>34</v>
+      </c>
+      <c r="H82" t="s">
+        <v>13</v>
+      </c>
+      <c r="I82" t="s">
+        <v>12</v>
+      </c>
+      <c r="J82">
+        <v>680</v>
+      </c>
+      <c r="K82">
+        <v>0</v>
+      </c>
+      <c r="L82">
+        <v>1</v>
+      </c>
+      <c r="M82">
+        <v>1</v>
+      </c>
+      <c r="N82">
+        <v>1</v>
+      </c>
+      <c r="O82">
+        <v>16</v>
+      </c>
+      <c r="P82">
+        <v>3</v>
+      </c>
+      <c r="Q82">
+        <v>12</v>
+      </c>
+      <c r="S82">
+        <v>4</v>
+      </c>
+      <c r="T82">
+        <v>20</v>
+      </c>
+      <c r="V82">
+        <v>8</v>
+      </c>
+      <c r="Z82">
+        <v>33</v>
+      </c>
+      <c r="AA82">
+        <v>3</v>
+      </c>
+      <c r="AB82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>23</v>
+      </c>
+      <c r="B83">
+        <v>2026</v>
+      </c>
+      <c r="C83">
+        <v>9</v>
+      </c>
+      <c r="D83">
+        <v>2</v>
+      </c>
+      <c r="E83">
+        <v>9</v>
+      </c>
+      <c r="F83">
+        <v>3</v>
+      </c>
+      <c r="G83" t="s">
+        <v>34</v>
+      </c>
+      <c r="H83" t="s">
+        <v>13</v>
+      </c>
+      <c r="I83" t="s">
+        <v>12</v>
+      </c>
+      <c r="J83">
+        <v>680</v>
+      </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
+      <c r="L83">
+        <v>1</v>
+      </c>
+      <c r="M83">
+        <v>1</v>
+      </c>
+      <c r="N83">
+        <v>1</v>
+      </c>
+      <c r="O83">
+        <v>17</v>
+      </c>
+      <c r="P83">
+        <v>3</v>
+      </c>
+      <c r="Q83">
+        <v>13</v>
+      </c>
+      <c r="S83">
+        <v>4</v>
+      </c>
+      <c r="U83">
+        <v>13</v>
+      </c>
+      <c r="V83">
+        <v>11</v>
+      </c>
+      <c r="Z83">
+        <v>35</v>
+      </c>
+      <c r="AA83">
+        <v>3</v>
+      </c>
+      <c r="AB83">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update w/ ipsos (9/13) and harris (9/14) polls
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF229AB-8246-E246-BDEE-540E7AF3F4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B41B771-1AFB-2D45-AC22-0E54C715E69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4380" yWindow="6700" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
+    <workbookView xWindow="340" yWindow="6860" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="41">
   <si>
     <t>id</t>
   </si>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AB83"/>
+  <dimension ref="A1:AB91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -6736,6 +6736,598 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>24</v>
+      </c>
+      <c r="B84">
+        <v>2026</v>
+      </c>
+      <c r="C84">
+        <v>9</v>
+      </c>
+      <c r="D84">
+        <v>8</v>
+      </c>
+      <c r="E84">
+        <v>9</v>
+      </c>
+      <c r="F84">
+        <v>9</v>
+      </c>
+      <c r="G84" t="s">
+        <v>34</v>
+      </c>
+      <c r="H84" t="s">
+        <v>13</v>
+      </c>
+      <c r="I84" t="s">
+        <v>12</v>
+      </c>
+      <c r="J84">
+        <v>699</v>
+      </c>
+      <c r="K84">
+        <v>0</v>
+      </c>
+      <c r="L84">
+        <v>1</v>
+      </c>
+      <c r="M84">
+        <v>1</v>
+      </c>
+      <c r="N84">
+        <v>1</v>
+      </c>
+      <c r="O84">
+        <v>15</v>
+      </c>
+      <c r="P84">
+        <v>2</v>
+      </c>
+      <c r="Q84">
+        <v>12</v>
+      </c>
+      <c r="S84">
+        <v>4</v>
+      </c>
+      <c r="U84">
+        <v>14</v>
+      </c>
+      <c r="V84">
+        <v>12</v>
+      </c>
+      <c r="X84">
+        <v>2</v>
+      </c>
+      <c r="Z84">
+        <v>34</v>
+      </c>
+      <c r="AA84">
+        <v>4</v>
+      </c>
+      <c r="AB84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>24</v>
+      </c>
+      <c r="B85">
+        <v>2026</v>
+      </c>
+      <c r="C85">
+        <v>9</v>
+      </c>
+      <c r="D85">
+        <v>8</v>
+      </c>
+      <c r="E85">
+        <v>9</v>
+      </c>
+      <c r="F85">
+        <v>9</v>
+      </c>
+      <c r="G85" t="s">
+        <v>34</v>
+      </c>
+      <c r="H85" t="s">
+        <v>13</v>
+      </c>
+      <c r="I85" t="s">
+        <v>12</v>
+      </c>
+      <c r="J85">
+        <v>699</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85">
+        <v>1</v>
+      </c>
+      <c r="M85">
+        <v>1</v>
+      </c>
+      <c r="N85">
+        <v>1</v>
+      </c>
+      <c r="O85">
+        <v>15</v>
+      </c>
+      <c r="P85">
+        <v>1</v>
+      </c>
+      <c r="Q85">
+        <v>10</v>
+      </c>
+      <c r="S85">
+        <v>3</v>
+      </c>
+      <c r="T85">
+        <v>19</v>
+      </c>
+      <c r="V85">
+        <v>10</v>
+      </c>
+      <c r="X85">
+        <v>3</v>
+      </c>
+      <c r="Z85">
+        <v>34</v>
+      </c>
+      <c r="AA85">
+        <v>4</v>
+      </c>
+      <c r="AB85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>25</v>
+      </c>
+      <c r="B86">
+        <v>2026</v>
+      </c>
+      <c r="C86">
+        <v>9</v>
+      </c>
+      <c r="D86">
+        <v>3</v>
+      </c>
+      <c r="E86">
+        <v>9</v>
+      </c>
+      <c r="F86">
+        <v>9</v>
+      </c>
+      <c r="G86" t="s">
+        <v>33</v>
+      </c>
+      <c r="H86" t="s">
+        <v>13</v>
+      </c>
+      <c r="I86" t="s">
+        <v>12</v>
+      </c>
+      <c r="J86">
+        <v>8488</v>
+      </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
+      <c r="L86">
+        <v>1</v>
+      </c>
+      <c r="M86">
+        <v>0.5</v>
+      </c>
+      <c r="N86">
+        <v>0.5</v>
+      </c>
+      <c r="O86">
+        <v>15.5</v>
+      </c>
+      <c r="P86">
+        <v>2.5</v>
+      </c>
+      <c r="Q86">
+        <v>12.5</v>
+      </c>
+      <c r="S86">
+        <v>4</v>
+      </c>
+      <c r="T86">
+        <v>17.5</v>
+      </c>
+      <c r="V86">
+        <v>8</v>
+      </c>
+      <c r="X86">
+        <v>2</v>
+      </c>
+      <c r="Z86">
+        <v>33.5</v>
+      </c>
+      <c r="AA86">
+        <v>4</v>
+      </c>
+      <c r="AB86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>25</v>
+      </c>
+      <c r="B87">
+        <v>2026</v>
+      </c>
+      <c r="C87">
+        <v>9</v>
+      </c>
+      <c r="D87">
+        <v>3</v>
+      </c>
+      <c r="E87">
+        <v>9</v>
+      </c>
+      <c r="F87">
+        <v>9</v>
+      </c>
+      <c r="G87" t="s">
+        <v>33</v>
+      </c>
+      <c r="H87" t="s">
+        <v>13</v>
+      </c>
+      <c r="I87" t="s">
+        <v>12</v>
+      </c>
+      <c r="J87">
+        <v>8310</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87">
+        <v>1</v>
+      </c>
+      <c r="M87">
+        <v>0.5</v>
+      </c>
+      <c r="N87">
+        <v>0.5</v>
+      </c>
+      <c r="O87">
+        <v>15.5</v>
+      </c>
+      <c r="P87">
+        <v>2.5</v>
+      </c>
+      <c r="Q87">
+        <v>13.5</v>
+      </c>
+      <c r="S87">
+        <v>4.5</v>
+      </c>
+      <c r="U87">
+        <v>13</v>
+      </c>
+      <c r="V87">
+        <v>10</v>
+      </c>
+      <c r="X87">
+        <v>2</v>
+      </c>
+      <c r="Z87">
+        <v>34</v>
+      </c>
+      <c r="AA87">
+        <v>4.5</v>
+      </c>
+      <c r="AB87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>26</v>
+      </c>
+      <c r="B88">
+        <v>2026</v>
+      </c>
+      <c r="C88">
+        <v>9</v>
+      </c>
+      <c r="D88">
+        <v>8</v>
+      </c>
+      <c r="E88">
+        <v>9</v>
+      </c>
+      <c r="F88">
+        <v>10</v>
+      </c>
+      <c r="G88" t="s">
+        <v>31</v>
+      </c>
+      <c r="H88" t="s">
+        <v>32</v>
+      </c>
+      <c r="I88" t="s">
+        <v>12</v>
+      </c>
+      <c r="J88">
+        <v>1765</v>
+      </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88">
+        <v>1</v>
+      </c>
+      <c r="M88">
+        <v>1</v>
+      </c>
+      <c r="N88">
+        <v>1</v>
+      </c>
+      <c r="O88">
+        <v>17</v>
+      </c>
+      <c r="P88">
+        <v>3</v>
+      </c>
+      <c r="Q88">
+        <v>10</v>
+      </c>
+      <c r="S88">
+        <v>3</v>
+      </c>
+      <c r="T88">
+        <v>17</v>
+      </c>
+      <c r="V88">
+        <v>7</v>
+      </c>
+      <c r="X88">
+        <v>3</v>
+      </c>
+      <c r="Z88">
+        <v>34</v>
+      </c>
+      <c r="AA88">
+        <v>5</v>
+      </c>
+      <c r="AB88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>26</v>
+      </c>
+      <c r="B89">
+        <v>2026</v>
+      </c>
+      <c r="C89">
+        <v>9</v>
+      </c>
+      <c r="D89">
+        <v>8</v>
+      </c>
+      <c r="E89">
+        <v>9</v>
+      </c>
+      <c r="F89">
+        <v>10</v>
+      </c>
+      <c r="G89" t="s">
+        <v>31</v>
+      </c>
+      <c r="H89" t="s">
+        <v>32</v>
+      </c>
+      <c r="I89" t="s">
+        <v>12</v>
+      </c>
+      <c r="J89">
+        <v>1744</v>
+      </c>
+      <c r="K89">
+        <v>0</v>
+      </c>
+      <c r="L89">
+        <v>1</v>
+      </c>
+      <c r="M89">
+        <v>1</v>
+      </c>
+      <c r="N89">
+        <v>1</v>
+      </c>
+      <c r="O89">
+        <v>17</v>
+      </c>
+      <c r="P89">
+        <v>2</v>
+      </c>
+      <c r="Q89">
+        <v>12</v>
+      </c>
+      <c r="S89">
+        <v>3</v>
+      </c>
+      <c r="U89">
+        <v>14</v>
+      </c>
+      <c r="V89">
+        <v>9</v>
+      </c>
+      <c r="X89">
+        <v>2</v>
+      </c>
+      <c r="Z89">
+        <v>35</v>
+      </c>
+      <c r="AA89">
+        <v>5</v>
+      </c>
+      <c r="AB89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>26</v>
+      </c>
+      <c r="B90">
+        <v>2026</v>
+      </c>
+      <c r="C90">
+        <v>9</v>
+      </c>
+      <c r="D90">
+        <v>8</v>
+      </c>
+      <c r="E90">
+        <v>9</v>
+      </c>
+      <c r="F90">
+        <v>10</v>
+      </c>
+      <c r="G90" t="s">
+        <v>31</v>
+      </c>
+      <c r="H90" t="s">
+        <v>32</v>
+      </c>
+      <c r="I90" t="s">
+        <v>12</v>
+      </c>
+      <c r="J90">
+        <v>1724</v>
+      </c>
+      <c r="K90">
+        <v>0</v>
+      </c>
+      <c r="L90">
+        <v>1</v>
+      </c>
+      <c r="M90">
+        <v>1</v>
+      </c>
+      <c r="N90">
+        <v>1</v>
+      </c>
+      <c r="O90">
+        <v>17</v>
+      </c>
+      <c r="P90">
+        <v>3</v>
+      </c>
+      <c r="R90">
+        <v>7</v>
+      </c>
+      <c r="S90">
+        <v>4</v>
+      </c>
+      <c r="T90">
+        <v>19</v>
+      </c>
+      <c r="V90">
+        <v>9</v>
+      </c>
+      <c r="X90">
+        <v>2</v>
+      </c>
+      <c r="Z90">
+        <v>33</v>
+      </c>
+      <c r="AA90">
+        <v>5</v>
+      </c>
+      <c r="AB90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>26</v>
+      </c>
+      <c r="B91">
+        <v>2026</v>
+      </c>
+      <c r="C91">
+        <v>9</v>
+      </c>
+      <c r="D91">
+        <v>8</v>
+      </c>
+      <c r="E91">
+        <v>9</v>
+      </c>
+      <c r="F91">
+        <v>10</v>
+      </c>
+      <c r="G91" t="s">
+        <v>31</v>
+      </c>
+      <c r="H91" t="s">
+        <v>32</v>
+      </c>
+      <c r="I91" t="s">
+        <v>12</v>
+      </c>
+      <c r="J91">
+        <v>1724</v>
+      </c>
+      <c r="K91">
+        <v>0</v>
+      </c>
+      <c r="L91">
+        <v>1</v>
+      </c>
+      <c r="M91">
+        <v>1</v>
+      </c>
+      <c r="N91">
+        <v>1</v>
+      </c>
+      <c r="O91">
+        <v>17</v>
+      </c>
+      <c r="P91">
+        <v>3</v>
+      </c>
+      <c r="R91">
+        <v>7</v>
+      </c>
+      <c r="S91">
+        <v>4</v>
+      </c>
+      <c r="U91">
+        <v>15</v>
+      </c>
+      <c r="V91">
+        <v>10</v>
+      </c>
+      <c r="X91">
+        <v>2</v>
+      </c>
+      <c r="Z91">
+        <v>36</v>
+      </c>
+      <c r="AA91">
+        <v>5</v>
+      </c>
+      <c r="AB91">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update with cluster17 (9/16) and harris (9/24) polls
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B41B771-1AFB-2D45-AC22-0E54C715E69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B5AEEC0-2C92-F74F-81E4-E00E1BC3971D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="6860" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
+    <workbookView xWindow="39040" yWindow="-800" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="41">
   <si>
     <t>id</t>
   </si>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AB91"/>
+  <dimension ref="A1:AB98"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -7328,6 +7328,518 @@
         <v>0</v>
       </c>
     </row>
+    <row r="92" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>27</v>
+      </c>
+      <c r="B92">
+        <v>2026</v>
+      </c>
+      <c r="C92">
+        <v>9</v>
+      </c>
+      <c r="D92">
+        <v>15</v>
+      </c>
+      <c r="E92">
+        <v>9</v>
+      </c>
+      <c r="F92">
+        <v>16</v>
+      </c>
+      <c r="G92" t="s">
+        <v>40</v>
+      </c>
+      <c r="H92" t="s">
+        <v>32</v>
+      </c>
+      <c r="I92" t="s">
+        <v>12</v>
+      </c>
+      <c r="J92">
+        <v>1733</v>
+      </c>
+      <c r="K92">
+        <v>0</v>
+      </c>
+      <c r="L92">
+        <v>1</v>
+      </c>
+      <c r="M92">
+        <v>0.1</v>
+      </c>
+      <c r="N92">
+        <v>0.4</v>
+      </c>
+      <c r="O92">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="P92">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="Q92">
+        <v>11.8</v>
+      </c>
+      <c r="S92">
+        <v>2.6</v>
+      </c>
+      <c r="T92">
+        <v>18.8</v>
+      </c>
+      <c r="V92">
+        <v>7.6</v>
+      </c>
+      <c r="X92">
+        <v>3.2</v>
+      </c>
+      <c r="Z92">
+        <v>30.8</v>
+      </c>
+      <c r="AA92">
+        <v>3.5</v>
+      </c>
+      <c r="AB92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>27</v>
+      </c>
+      <c r="B93">
+        <v>2026</v>
+      </c>
+      <c r="C93">
+        <v>9</v>
+      </c>
+      <c r="D93">
+        <v>15</v>
+      </c>
+      <c r="E93">
+        <v>9</v>
+      </c>
+      <c r="F93">
+        <v>16</v>
+      </c>
+      <c r="G93" t="s">
+        <v>40</v>
+      </c>
+      <c r="H93" t="s">
+        <v>32</v>
+      </c>
+      <c r="I93" t="s">
+        <v>12</v>
+      </c>
+      <c r="J93">
+        <v>1723</v>
+      </c>
+      <c r="K93">
+        <v>0</v>
+      </c>
+      <c r="L93">
+        <v>1</v>
+      </c>
+      <c r="M93">
+        <v>0.1</v>
+      </c>
+      <c r="N93">
+        <v>0.4</v>
+      </c>
+      <c r="O93">
+        <v>19.8</v>
+      </c>
+      <c r="P93">
+        <v>2.5</v>
+      </c>
+      <c r="Q93">
+        <v>14</v>
+      </c>
+      <c r="S93">
+        <v>2.6</v>
+      </c>
+      <c r="U93">
+        <v>13.4</v>
+      </c>
+      <c r="V93">
+        <v>9.5</v>
+      </c>
+      <c r="X93">
+        <v>3.2</v>
+      </c>
+      <c r="Z93">
+        <v>31</v>
+      </c>
+      <c r="AA93">
+        <v>3.6</v>
+      </c>
+      <c r="AB93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>27</v>
+      </c>
+      <c r="B94">
+        <v>2026</v>
+      </c>
+      <c r="C94">
+        <v>9</v>
+      </c>
+      <c r="D94">
+        <v>15</v>
+      </c>
+      <c r="E94">
+        <v>9</v>
+      </c>
+      <c r="F94">
+        <v>16</v>
+      </c>
+      <c r="G94" t="s">
+        <v>40</v>
+      </c>
+      <c r="H94" t="s">
+        <v>32</v>
+      </c>
+      <c r="I94" t="s">
+        <v>12</v>
+      </c>
+      <c r="J94">
+        <v>1729</v>
+      </c>
+      <c r="K94">
+        <v>0</v>
+      </c>
+      <c r="L94">
+        <v>1</v>
+      </c>
+      <c r="M94">
+        <v>0.1</v>
+      </c>
+      <c r="N94">
+        <v>0.7</v>
+      </c>
+      <c r="O94">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="P94">
+        <v>2.9</v>
+      </c>
+      <c r="R94">
+        <v>7.4</v>
+      </c>
+      <c r="S94">
+        <v>3</v>
+      </c>
+      <c r="T94">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="V94">
+        <v>7.6</v>
+      </c>
+      <c r="X94">
+        <v>4</v>
+      </c>
+      <c r="Z94">
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>28</v>
+      </c>
+      <c r="B95">
+        <v>2026</v>
+      </c>
+      <c r="C95">
+        <v>9</v>
+      </c>
+      <c r="D95">
+        <v>22</v>
+      </c>
+      <c r="E95">
+        <v>9</v>
+      </c>
+      <c r="F95">
+        <v>24</v>
+      </c>
+      <c r="G95" t="s">
+        <v>31</v>
+      </c>
+      <c r="H95" t="s">
+        <v>32</v>
+      </c>
+      <c r="I95" t="s">
+        <v>12</v>
+      </c>
+      <c r="J95">
+        <v>1678</v>
+      </c>
+      <c r="K95">
+        <v>0</v>
+      </c>
+      <c r="L95">
+        <v>1</v>
+      </c>
+      <c r="M95">
+        <v>1</v>
+      </c>
+      <c r="N95">
+        <v>1</v>
+      </c>
+      <c r="O95">
+        <v>18</v>
+      </c>
+      <c r="P95">
+        <v>2</v>
+      </c>
+      <c r="Q95">
+        <v>10</v>
+      </c>
+      <c r="S95">
+        <v>3</v>
+      </c>
+      <c r="T95">
+        <v>16</v>
+      </c>
+      <c r="V95">
+        <v>8</v>
+      </c>
+      <c r="X95">
+        <v>2</v>
+      </c>
+      <c r="Z95">
+        <v>35</v>
+      </c>
+      <c r="AA95">
+        <v>5</v>
+      </c>
+      <c r="AB95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>28</v>
+      </c>
+      <c r="B96">
+        <v>2026</v>
+      </c>
+      <c r="C96">
+        <v>9</v>
+      </c>
+      <c r="D96">
+        <v>22</v>
+      </c>
+      <c r="E96">
+        <v>9</v>
+      </c>
+      <c r="F96">
+        <v>24</v>
+      </c>
+      <c r="G96" t="s">
+        <v>31</v>
+      </c>
+      <c r="H96" t="s">
+        <v>32</v>
+      </c>
+      <c r="I96" t="s">
+        <v>12</v>
+      </c>
+      <c r="J96">
+        <v>1638</v>
+      </c>
+      <c r="K96">
+        <v>0</v>
+      </c>
+      <c r="L96">
+        <v>1</v>
+      </c>
+      <c r="M96">
+        <v>1</v>
+      </c>
+      <c r="N96">
+        <v>1</v>
+      </c>
+      <c r="O96">
+        <v>17</v>
+      </c>
+      <c r="P96">
+        <v>2</v>
+      </c>
+      <c r="Q96">
+        <v>11</v>
+      </c>
+      <c r="S96">
+        <v>3</v>
+      </c>
+      <c r="U96">
+        <v>12</v>
+      </c>
+      <c r="V96">
+        <v>10</v>
+      </c>
+      <c r="X96">
+        <v>2</v>
+      </c>
+      <c r="Z96">
+        <v>36</v>
+      </c>
+      <c r="AA96">
+        <v>6</v>
+      </c>
+      <c r="AB96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>28</v>
+      </c>
+      <c r="B97">
+        <v>2026</v>
+      </c>
+      <c r="C97">
+        <v>9</v>
+      </c>
+      <c r="D97">
+        <v>22</v>
+      </c>
+      <c r="E97">
+        <v>9</v>
+      </c>
+      <c r="F97">
+        <v>24</v>
+      </c>
+      <c r="G97" t="s">
+        <v>31</v>
+      </c>
+      <c r="H97" t="s">
+        <v>32</v>
+      </c>
+      <c r="I97" t="s">
+        <v>12</v>
+      </c>
+      <c r="J97">
+        <v>1658</v>
+      </c>
+      <c r="K97">
+        <v>0</v>
+      </c>
+      <c r="L97">
+        <v>1</v>
+      </c>
+      <c r="M97">
+        <v>1</v>
+      </c>
+      <c r="N97">
+        <v>1</v>
+      </c>
+      <c r="O97">
+        <v>18</v>
+      </c>
+      <c r="P97">
+        <v>3</v>
+      </c>
+      <c r="R97">
+        <v>7</v>
+      </c>
+      <c r="S97">
+        <v>4</v>
+      </c>
+      <c r="T97">
+        <v>16</v>
+      </c>
+      <c r="V97">
+        <v>9</v>
+      </c>
+      <c r="X97">
+        <v>2</v>
+      </c>
+      <c r="Z97">
+        <v>35</v>
+      </c>
+      <c r="AA97">
+        <v>5</v>
+      </c>
+      <c r="AB97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>28</v>
+      </c>
+      <c r="B98">
+        <v>2026</v>
+      </c>
+      <c r="C98">
+        <v>9</v>
+      </c>
+      <c r="D98">
+        <v>22</v>
+      </c>
+      <c r="E98">
+        <v>9</v>
+      </c>
+      <c r="F98">
+        <v>24</v>
+      </c>
+      <c r="G98" t="s">
+        <v>31</v>
+      </c>
+      <c r="H98" t="s">
+        <v>32</v>
+      </c>
+      <c r="I98" t="s">
+        <v>12</v>
+      </c>
+      <c r="J98">
+        <v>1638</v>
+      </c>
+      <c r="K98">
+        <v>0</v>
+      </c>
+      <c r="L98">
+        <v>1</v>
+      </c>
+      <c r="M98">
+        <v>1</v>
+      </c>
+      <c r="N98">
+        <v>1</v>
+      </c>
+      <c r="O98">
+        <v>17</v>
+      </c>
+      <c r="P98">
+        <v>3</v>
+      </c>
+      <c r="R98">
+        <v>8</v>
+      </c>
+      <c r="S98">
+        <v>5</v>
+      </c>
+      <c r="U98">
+        <v>13</v>
+      </c>
+      <c r="V98">
+        <v>10</v>
+      </c>
+      <c r="X98">
+        <v>2</v>
+      </c>
+      <c r="Z98">
+        <v>36</v>
+      </c>
+      <c r="AA98">
+        <v>5</v>
+      </c>
+      <c r="AB98">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update w/ harris (10/8), ow (10/14), odoxa (10/7)
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B5AEEC0-2C92-F74F-81E4-E00E1BC3971D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F50F45D-E9D1-CB45-97CA-0B96F01BEE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39040" yWindow="-800" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
+    <workbookView xWindow="39040" yWindow="-940" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="41">
   <si>
     <t>id</t>
   </si>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AB98"/>
+  <dimension ref="A1:AB106"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -7543,6 +7543,9 @@
       <c r="Z94">
         <v>30.2</v>
       </c>
+      <c r="AB94">
+        <v>0</v>
+      </c>
     </row>
     <row r="95" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A95">
@@ -7837,6 +7840,598 @@
         <v>5</v>
       </c>
       <c r="AB98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>29</v>
+      </c>
+      <c r="B99">
+        <v>2026</v>
+      </c>
+      <c r="C99">
+        <v>10</v>
+      </c>
+      <c r="D99">
+        <v>5</v>
+      </c>
+      <c r="E99">
+        <v>10</v>
+      </c>
+      <c r="F99">
+        <v>8</v>
+      </c>
+      <c r="G99" t="s">
+        <v>31</v>
+      </c>
+      <c r="H99" t="s">
+        <v>32</v>
+      </c>
+      <c r="I99" t="s">
+        <v>12</v>
+      </c>
+      <c r="J99">
+        <v>1683</v>
+      </c>
+      <c r="K99">
+        <v>0</v>
+      </c>
+      <c r="L99">
+        <v>1</v>
+      </c>
+      <c r="M99">
+        <v>1</v>
+      </c>
+      <c r="N99">
+        <v>1</v>
+      </c>
+      <c r="O99">
+        <v>18</v>
+      </c>
+      <c r="P99">
+        <v>2</v>
+      </c>
+      <c r="Q99">
+        <v>10</v>
+      </c>
+      <c r="S99">
+        <v>3</v>
+      </c>
+      <c r="T99">
+        <v>17</v>
+      </c>
+      <c r="V99">
+        <v>7</v>
+      </c>
+      <c r="X99">
+        <v>2</v>
+      </c>
+      <c r="Z99">
+        <v>36</v>
+      </c>
+      <c r="AA99">
+        <v>4</v>
+      </c>
+      <c r="AB99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>29</v>
+      </c>
+      <c r="B100">
+        <v>2026</v>
+      </c>
+      <c r="C100">
+        <v>10</v>
+      </c>
+      <c r="D100">
+        <v>5</v>
+      </c>
+      <c r="E100">
+        <v>10</v>
+      </c>
+      <c r="F100">
+        <v>8</v>
+      </c>
+      <c r="G100" t="s">
+        <v>31</v>
+      </c>
+      <c r="H100" t="s">
+        <v>32</v>
+      </c>
+      <c r="I100" t="s">
+        <v>12</v>
+      </c>
+      <c r="J100">
+        <v>1663</v>
+      </c>
+      <c r="K100">
+        <v>0</v>
+      </c>
+      <c r="L100">
+        <v>1</v>
+      </c>
+      <c r="M100">
+        <v>1</v>
+      </c>
+      <c r="N100">
+        <v>1</v>
+      </c>
+      <c r="O100">
+        <v>18</v>
+      </c>
+      <c r="P100">
+        <v>2</v>
+      </c>
+      <c r="Q100">
+        <v>11</v>
+      </c>
+      <c r="S100">
+        <v>3</v>
+      </c>
+      <c r="U100">
+        <v>12</v>
+      </c>
+      <c r="V100">
+        <v>10</v>
+      </c>
+      <c r="X100">
+        <v>2</v>
+      </c>
+      <c r="Z100">
+        <v>36</v>
+      </c>
+      <c r="AA100">
+        <v>5</v>
+      </c>
+      <c r="AB100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>29</v>
+      </c>
+      <c r="B101">
+        <v>2026</v>
+      </c>
+      <c r="C101">
+        <v>10</v>
+      </c>
+      <c r="D101">
+        <v>5</v>
+      </c>
+      <c r="E101">
+        <v>10</v>
+      </c>
+      <c r="F101">
+        <v>8</v>
+      </c>
+      <c r="G101" t="s">
+        <v>31</v>
+      </c>
+      <c r="H101" t="s">
+        <v>32</v>
+      </c>
+      <c r="I101" t="s">
+        <v>12</v>
+      </c>
+      <c r="J101">
+        <v>1643</v>
+      </c>
+      <c r="K101">
+        <v>0</v>
+      </c>
+      <c r="L101">
+        <v>1</v>
+      </c>
+      <c r="M101">
+        <v>1</v>
+      </c>
+      <c r="N101">
+        <v>1</v>
+      </c>
+      <c r="O101">
+        <v>18</v>
+      </c>
+      <c r="P101">
+        <v>3</v>
+      </c>
+      <c r="R101">
+        <v>7</v>
+      </c>
+      <c r="S101">
+        <v>4</v>
+      </c>
+      <c r="T101">
+        <v>17</v>
+      </c>
+      <c r="V101">
+        <v>8</v>
+      </c>
+      <c r="X101">
+        <v>2</v>
+      </c>
+      <c r="Z101">
+        <v>36</v>
+      </c>
+      <c r="AA101">
+        <v>4</v>
+      </c>
+      <c r="AB101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>29</v>
+      </c>
+      <c r="B102">
+        <v>2026</v>
+      </c>
+      <c r="C102">
+        <v>10</v>
+      </c>
+      <c r="D102">
+        <v>5</v>
+      </c>
+      <c r="E102">
+        <v>10</v>
+      </c>
+      <c r="F102">
+        <v>8</v>
+      </c>
+      <c r="G102" t="s">
+        <v>31</v>
+      </c>
+      <c r="H102" t="s">
+        <v>32</v>
+      </c>
+      <c r="I102" t="s">
+        <v>12</v>
+      </c>
+      <c r="J102">
+        <v>1663</v>
+      </c>
+      <c r="K102">
+        <v>0</v>
+      </c>
+      <c r="L102">
+        <v>1</v>
+      </c>
+      <c r="M102">
+        <v>1</v>
+      </c>
+      <c r="N102">
+        <v>1</v>
+      </c>
+      <c r="O102">
+        <v>19</v>
+      </c>
+      <c r="P102">
+        <v>2</v>
+      </c>
+      <c r="R102">
+        <v>7</v>
+      </c>
+      <c r="S102">
+        <v>5</v>
+      </c>
+      <c r="U102">
+        <v>12</v>
+      </c>
+      <c r="V102">
+        <v>10</v>
+      </c>
+      <c r="X102">
+        <v>2</v>
+      </c>
+      <c r="Z102">
+        <v>37</v>
+      </c>
+      <c r="AA102">
+        <v>5</v>
+      </c>
+      <c r="AB102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>30</v>
+      </c>
+      <c r="B103">
+        <v>2026</v>
+      </c>
+      <c r="C103">
+        <v>10</v>
+      </c>
+      <c r="D103">
+        <v>13</v>
+      </c>
+      <c r="E103">
+        <v>10</v>
+      </c>
+      <c r="F103">
+        <v>14</v>
+      </c>
+      <c r="G103" t="s">
+        <v>34</v>
+      </c>
+      <c r="H103" t="s">
+        <v>13</v>
+      </c>
+      <c r="I103" t="s">
+        <v>12</v>
+      </c>
+      <c r="J103">
+        <v>731</v>
+      </c>
+      <c r="K103">
+        <v>0</v>
+      </c>
+      <c r="L103">
+        <v>1</v>
+      </c>
+      <c r="M103">
+        <v>1</v>
+      </c>
+      <c r="N103">
+        <v>1</v>
+      </c>
+      <c r="O103">
+        <v>15</v>
+      </c>
+      <c r="P103">
+        <v>2</v>
+      </c>
+      <c r="Q103">
+        <v>16</v>
+      </c>
+      <c r="S103">
+        <v>3</v>
+      </c>
+      <c r="U103">
+        <v>11</v>
+      </c>
+      <c r="V103">
+        <v>9</v>
+      </c>
+      <c r="X103">
+        <v>2</v>
+      </c>
+      <c r="Z103">
+        <v>37</v>
+      </c>
+      <c r="AA103">
+        <v>4</v>
+      </c>
+      <c r="AB103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>30</v>
+      </c>
+      <c r="B104">
+        <v>2026</v>
+      </c>
+      <c r="C104">
+        <v>10</v>
+      </c>
+      <c r="D104">
+        <v>13</v>
+      </c>
+      <c r="E104">
+        <v>10</v>
+      </c>
+      <c r="F104">
+        <v>14</v>
+      </c>
+      <c r="G104" t="s">
+        <v>34</v>
+      </c>
+      <c r="H104" t="s">
+        <v>13</v>
+      </c>
+      <c r="I104" t="s">
+        <v>12</v>
+      </c>
+      <c r="J104">
+        <v>731</v>
+      </c>
+      <c r="K104">
+        <v>0</v>
+      </c>
+      <c r="L104">
+        <v>1</v>
+      </c>
+      <c r="M104">
+        <v>1</v>
+      </c>
+      <c r="N104">
+        <v>1</v>
+      </c>
+      <c r="O104">
+        <v>15</v>
+      </c>
+      <c r="P104">
+        <v>2</v>
+      </c>
+      <c r="Q104">
+        <v>15</v>
+      </c>
+      <c r="S104">
+        <v>3</v>
+      </c>
+      <c r="T104">
+        <v>15</v>
+      </c>
+      <c r="V104">
+        <v>8</v>
+      </c>
+      <c r="X104">
+        <v>2</v>
+      </c>
+      <c r="Z104">
+        <v>35</v>
+      </c>
+      <c r="AA104">
+        <v>4</v>
+      </c>
+      <c r="AB104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <v>31</v>
+      </c>
+      <c r="B105">
+        <v>2026</v>
+      </c>
+      <c r="C105">
+        <v>9</v>
+      </c>
+      <c r="D105">
+        <v>24</v>
+      </c>
+      <c r="E105">
+        <v>10</v>
+      </c>
+      <c r="F105">
+        <v>7</v>
+      </c>
+      <c r="G105" t="s">
+        <v>27</v>
+      </c>
+      <c r="H105" t="s">
+        <v>28</v>
+      </c>
+      <c r="I105" t="s">
+        <v>12</v>
+      </c>
+      <c r="J105">
+        <v>7599</v>
+      </c>
+      <c r="K105">
+        <v>0</v>
+      </c>
+      <c r="L105">
+        <v>1</v>
+      </c>
+      <c r="M105">
+        <v>0.5</v>
+      </c>
+      <c r="N105">
+        <v>0.5</v>
+      </c>
+      <c r="O105">
+        <v>18</v>
+      </c>
+      <c r="P105">
+        <v>2</v>
+      </c>
+      <c r="Q105">
+        <v>9.5</v>
+      </c>
+      <c r="S105">
+        <v>3</v>
+      </c>
+      <c r="T105">
+        <v>17</v>
+      </c>
+      <c r="V105">
+        <v>6.5</v>
+      </c>
+      <c r="X105">
+        <v>2</v>
+      </c>
+      <c r="Z105">
+        <v>37</v>
+      </c>
+      <c r="AA105">
+        <v>4.5</v>
+      </c>
+      <c r="AB105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <v>31</v>
+      </c>
+      <c r="B106">
+        <v>2026</v>
+      </c>
+      <c r="C106">
+        <v>9</v>
+      </c>
+      <c r="D106">
+        <v>24</v>
+      </c>
+      <c r="E106">
+        <v>10</v>
+      </c>
+      <c r="F106">
+        <v>7</v>
+      </c>
+      <c r="G106" t="s">
+        <v>27</v>
+      </c>
+      <c r="H106" t="s">
+        <v>28</v>
+      </c>
+      <c r="I106" t="s">
+        <v>12</v>
+      </c>
+      <c r="J106">
+        <v>7374</v>
+      </c>
+      <c r="K106">
+        <v>0</v>
+      </c>
+      <c r="L106">
+        <v>1</v>
+      </c>
+      <c r="M106">
+        <v>0.5</v>
+      </c>
+      <c r="N106">
+        <v>1</v>
+      </c>
+      <c r="O106">
+        <v>18.5</v>
+      </c>
+      <c r="P106">
+        <v>2</v>
+      </c>
+      <c r="Q106">
+        <v>10.5</v>
+      </c>
+      <c r="S106">
+        <v>3.5</v>
+      </c>
+      <c r="U106">
+        <v>11</v>
+      </c>
+      <c r="V106">
+        <v>9</v>
+      </c>
+      <c r="X106">
+        <v>2</v>
+      </c>
+      <c r="Z106">
+        <v>38</v>
+      </c>
+      <c r="AA106">
+        <v>4.5</v>
+      </c>
+      <c r="AB106">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update w/ ifop (10/13), elabe (10/14), yougov (10/15)
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F50F45D-E9D1-CB45-97CA-0B96F01BEE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3544FDE-0139-F94E-AC96-C927371347F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39040" yWindow="-940" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
+    <workbookView xWindow="35620" yWindow="14060" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -162,6 +162,12 @@
   </si>
   <si>
     <t>cluster17</t>
+  </si>
+  <si>
+    <t>c_lisnard</t>
+  </si>
+  <si>
+    <t>yougov</t>
   </si>
 </sst>
 </file>
@@ -561,13 +567,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AB106"/>
+  <dimension ref="A1:AC113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -632,28 +638,31 @@
         <v>20</v>
       </c>
       <c r="V1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -711,26 +720,26 @@
       <c r="T2">
         <v>16</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>10</v>
       </c>
-      <c r="W2">
+      <c r="X2">
         <v>3.5</v>
       </c>
-      <c r="X2">
+      <c r="Y2">
         <v>2.5</v>
       </c>
-      <c r="Y2">
+      <c r="Z2">
         <v>36</v>
       </c>
-      <c r="AA2">
-        <v>4</v>
-      </c>
       <c r="AB2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -788,26 +797,26 @@
       <c r="T3">
         <v>16</v>
       </c>
-      <c r="V3">
+      <c r="W3">
         <v>11</v>
       </c>
-      <c r="W3">
+      <c r="X3">
         <v>5</v>
       </c>
-      <c r="X3">
-        <v>2</v>
-      </c>
-      <c r="Z3">
+      <c r="Y3">
+        <v>2</v>
+      </c>
+      <c r="AA3">
         <v>34</v>
       </c>
-      <c r="AA3">
-        <v>4</v>
-      </c>
       <c r="AB3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -865,26 +874,26 @@
       <c r="U4">
         <v>11</v>
       </c>
-      <c r="V4">
-        <v>12</v>
-      </c>
       <c r="W4">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="X4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y4">
+        <v>2</v>
+      </c>
+      <c r="Z4">
         <v>36</v>
       </c>
-      <c r="AA4">
-        <v>4</v>
-      </c>
       <c r="AB4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -942,26 +951,26 @@
       <c r="U5">
         <v>10</v>
       </c>
-      <c r="V5">
-        <v>12</v>
-      </c>
       <c r="W5">
+        <v>12</v>
+      </c>
+      <c r="X5">
         <v>4.5</v>
       </c>
-      <c r="X5">
-        <v>3</v>
-      </c>
-      <c r="Z5">
+      <c r="Y5">
+        <v>3</v>
+      </c>
+      <c r="AA5">
         <v>35</v>
       </c>
-      <c r="AA5">
-        <v>4</v>
-      </c>
       <c r="AB5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1019,23 +1028,23 @@
       <c r="T6">
         <v>21</v>
       </c>
-      <c r="V6">
-        <v>8</v>
-      </c>
-      <c r="X6">
-        <v>2</v>
+      <c r="W6">
+        <v>8</v>
       </c>
       <c r="Y6">
+        <v>2</v>
+      </c>
+      <c r="Z6">
         <v>34</v>
       </c>
-      <c r="AA6">
+      <c r="AB6">
         <v>5</v>
       </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2</v>
       </c>
@@ -1093,20 +1102,20 @@
       <c r="T7">
         <v>25</v>
       </c>
-      <c r="X7">
-        <v>2</v>
-      </c>
       <c r="Y7">
+        <v>2</v>
+      </c>
+      <c r="Z7">
         <v>38</v>
       </c>
-      <c r="AA7">
+      <c r="AB7">
         <v>5</v>
       </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>3</v>
       </c>
@@ -1164,26 +1173,26 @@
       <c r="T8">
         <v>20.5</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <v>7</v>
       </c>
-      <c r="W8">
-        <v>3</v>
-      </c>
       <c r="X8">
+        <v>3</v>
+      </c>
+      <c r="Y8">
         <v>2.5</v>
       </c>
-      <c r="Y8">
+      <c r="Z8">
         <v>35</v>
       </c>
-      <c r="AA8">
-        <v>3</v>
-      </c>
       <c r="AB8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1241,26 +1250,26 @@
       <c r="T9">
         <v>22</v>
       </c>
-      <c r="V9">
+      <c r="W9">
         <v>8.5</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <v>2.5</v>
       </c>
-      <c r="X9">
-        <v>3</v>
-      </c>
-      <c r="Z9">
+      <c r="Y9">
+        <v>3</v>
+      </c>
+      <c r="AA9">
         <v>31.5</v>
       </c>
-      <c r="AA9">
+      <c r="AB9">
         <v>3.5</v>
       </c>
-      <c r="AB9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>3</v>
       </c>
@@ -1318,26 +1327,26 @@
       <c r="U10">
         <v>11.5</v>
       </c>
-      <c r="V10">
+      <c r="W10">
         <v>10</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <v>6</v>
       </c>
-      <c r="X10">
+      <c r="Y10">
         <v>2.5</v>
       </c>
-      <c r="Z10">
+      <c r="AA10">
         <v>34</v>
       </c>
-      <c r="AA10">
-        <v>4</v>
-      </c>
       <c r="AB10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1395,23 +1404,23 @@
       <c r="T11">
         <v>18</v>
       </c>
-      <c r="V11">
+      <c r="W11">
         <v>7</v>
       </c>
-      <c r="X11">
-        <v>2</v>
-      </c>
       <c r="Y11">
+        <v>2</v>
+      </c>
+      <c r="Z11">
         <v>35</v>
       </c>
-      <c r="AA11">
+      <c r="AB11">
         <v>5</v>
       </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4</v>
       </c>
@@ -1469,23 +1478,23 @@
       <c r="U12">
         <v>13</v>
       </c>
-      <c r="V12">
+      <c r="W12">
         <v>10</v>
       </c>
-      <c r="X12">
-        <v>2</v>
-      </c>
       <c r="Y12">
+        <v>2</v>
+      </c>
+      <c r="Z12">
         <v>36</v>
       </c>
-      <c r="AA12">
+      <c r="AB12">
         <v>5</v>
       </c>
-      <c r="AB12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>5</v>
       </c>
@@ -1543,23 +1552,23 @@
       <c r="T13">
         <v>19</v>
       </c>
-      <c r="V13">
-        <v>9</v>
-      </c>
-      <c r="X13">
-        <v>1</v>
+      <c r="W13">
+        <v>9</v>
       </c>
       <c r="Y13">
+        <v>1</v>
+      </c>
+      <c r="Z13">
         <v>34</v>
       </c>
-      <c r="AA13">
+      <c r="AB13">
         <v>5</v>
       </c>
-      <c r="AB13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1617,23 +1626,23 @@
       <c r="U14">
         <v>14</v>
       </c>
-      <c r="V14">
-        <v>12</v>
-      </c>
-      <c r="X14">
-        <v>1</v>
+      <c r="W14">
+        <v>12</v>
       </c>
       <c r="Y14">
+        <v>1</v>
+      </c>
+      <c r="Z14">
         <v>35</v>
       </c>
-      <c r="AA14">
+      <c r="AB14">
         <v>5</v>
       </c>
-      <c r="AB14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>5</v>
       </c>
@@ -1691,23 +1700,23 @@
       <c r="T15">
         <v>19</v>
       </c>
-      <c r="V15">
+      <c r="W15">
         <v>10</v>
       </c>
-      <c r="X15">
-        <v>1</v>
-      </c>
-      <c r="Z15">
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="AA15">
         <v>32</v>
       </c>
-      <c r="AA15">
+      <c r="AB15">
         <v>6</v>
       </c>
-      <c r="AB15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>5</v>
       </c>
@@ -1765,23 +1774,23 @@
       <c r="U16">
         <v>14</v>
       </c>
-      <c r="V16">
-        <v>13</v>
-      </c>
-      <c r="X16">
-        <v>2</v>
-      </c>
-      <c r="Z16">
+      <c r="W16">
+        <v>13</v>
+      </c>
+      <c r="Y16">
+        <v>2</v>
+      </c>
+      <c r="AA16">
         <v>33</v>
       </c>
-      <c r="AA16">
+      <c r="AB16">
         <v>5</v>
       </c>
-      <c r="AB16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>6</v>
       </c>
@@ -1839,23 +1848,23 @@
       <c r="T17">
         <v>17</v>
       </c>
-      <c r="V17">
-        <v>9</v>
-      </c>
-      <c r="X17">
-        <v>2</v>
+      <c r="W17">
+        <v>9</v>
       </c>
       <c r="Y17">
+        <v>2</v>
+      </c>
+      <c r="Z17">
         <v>34</v>
       </c>
-      <c r="AA17">
+      <c r="AB17">
         <v>6</v>
       </c>
-      <c r="AB17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>7</v>
       </c>
@@ -1913,23 +1922,23 @@
       <c r="T18">
         <v>13</v>
       </c>
-      <c r="V18">
-        <v>8</v>
-      </c>
-      <c r="X18">
-        <v>2</v>
+      <c r="W18">
+        <v>8</v>
       </c>
       <c r="Y18">
+        <v>2</v>
+      </c>
+      <c r="Z18">
         <v>32</v>
       </c>
-      <c r="AA18">
+      <c r="AB18">
         <v>5</v>
       </c>
-      <c r="AB18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>7</v>
       </c>
@@ -1987,23 +1996,23 @@
       <c r="T19">
         <v>17</v>
       </c>
-      <c r="V19">
-        <v>9</v>
-      </c>
-      <c r="X19">
-        <v>2</v>
+      <c r="W19">
+        <v>9</v>
       </c>
       <c r="Y19">
+        <v>2</v>
+      </c>
+      <c r="Z19">
         <v>34</v>
       </c>
-      <c r="AA19">
+      <c r="AB19">
         <v>6</v>
       </c>
-      <c r="AB19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>7</v>
       </c>
@@ -2061,23 +2070,23 @@
       <c r="U20">
         <v>14</v>
       </c>
-      <c r="V20">
+      <c r="W20">
         <v>10</v>
       </c>
-      <c r="X20">
-        <v>2</v>
-      </c>
       <c r="Y20">
+        <v>2</v>
+      </c>
+      <c r="Z20">
         <v>34</v>
       </c>
-      <c r="AA20">
+      <c r="AB20">
         <v>6</v>
       </c>
-      <c r="AB20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>7</v>
       </c>
@@ -2135,23 +2144,23 @@
       <c r="T21">
         <v>19</v>
       </c>
-      <c r="V21">
+      <c r="W21">
         <v>10</v>
       </c>
-      <c r="X21">
-        <v>2</v>
-      </c>
-      <c r="Z21">
+      <c r="Y21">
+        <v>2</v>
+      </c>
+      <c r="AA21">
         <v>31</v>
       </c>
-      <c r="AA21">
+      <c r="AB21">
         <v>6</v>
       </c>
-      <c r="AB21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>7</v>
       </c>
@@ -2209,23 +2218,23 @@
       <c r="U22">
         <v>15</v>
       </c>
-      <c r="V22">
+      <c r="W22">
         <v>11</v>
       </c>
-      <c r="X22">
-        <v>2</v>
-      </c>
-      <c r="Z22">
+      <c r="Y22">
+        <v>2</v>
+      </c>
+      <c r="AA22">
         <v>32</v>
       </c>
-      <c r="AA22">
+      <c r="AB22">
         <v>6</v>
       </c>
-      <c r="AB22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>8</v>
       </c>
@@ -2286,23 +2295,23 @@
       <c r="U23">
         <v>9</v>
       </c>
-      <c r="V23">
-        <v>8</v>
-      </c>
-      <c r="X23">
-        <v>2</v>
+      <c r="W23">
+        <v>8</v>
       </c>
       <c r="Y23">
+        <v>2</v>
+      </c>
+      <c r="Z23">
         <v>34</v>
       </c>
-      <c r="AA23">
-        <v>4</v>
-      </c>
       <c r="AB23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>8</v>
       </c>
@@ -2360,26 +2369,26 @@
       <c r="T24">
         <v>18</v>
       </c>
-      <c r="V24">
-        <v>9</v>
-      </c>
       <c r="W24">
+        <v>9</v>
+      </c>
+      <c r="X24">
         <v>2.5</v>
       </c>
-      <c r="X24">
-        <v>2</v>
-      </c>
       <c r="Y24">
+        <v>2</v>
+      </c>
+      <c r="Z24">
         <v>34</v>
       </c>
-      <c r="AA24">
+      <c r="AB24">
         <v>3.5</v>
       </c>
-      <c r="AB24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>8</v>
       </c>
@@ -2437,26 +2446,26 @@
       <c r="U25">
         <v>16</v>
       </c>
-      <c r="V25">
+      <c r="W25">
         <v>10</v>
       </c>
-      <c r="W25">
-        <v>3</v>
-      </c>
       <c r="X25">
+        <v>3</v>
+      </c>
+      <c r="Y25">
         <v>2.5</v>
       </c>
-      <c r="Y25">
+      <c r="Z25">
         <v>34</v>
       </c>
-      <c r="AA25">
-        <v>3</v>
-      </c>
       <c r="AB25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>8</v>
       </c>
@@ -2514,26 +2523,26 @@
       <c r="T26">
         <v>19</v>
       </c>
-      <c r="V26">
-        <v>9</v>
-      </c>
       <c r="W26">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="X26">
+        <v>2</v>
+      </c>
+      <c r="Y26">
         <v>1.5</v>
       </c>
-      <c r="Z26">
+      <c r="AA26">
         <v>33</v>
       </c>
-      <c r="AA26">
-        <v>4</v>
-      </c>
       <c r="AB26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>8</v>
       </c>
@@ -2591,26 +2600,26 @@
       <c r="U27">
         <v>16</v>
       </c>
-      <c r="V27">
+      <c r="W27">
         <v>11.5</v>
       </c>
-      <c r="W27">
-        <v>3</v>
-      </c>
       <c r="X27">
-        <v>2</v>
-      </c>
-      <c r="Z27">
+        <v>3</v>
+      </c>
+      <c r="Y27">
+        <v>2</v>
+      </c>
+      <c r="AA27">
         <v>32</v>
       </c>
-      <c r="AA27">
-        <v>4</v>
-      </c>
       <c r="AB27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>8</v>
       </c>
@@ -2668,23 +2677,23 @@
       <c r="T28">
         <v>20</v>
       </c>
-      <c r="V28">
-        <v>9</v>
-      </c>
-      <c r="X28">
+      <c r="W28">
+        <v>9</v>
+      </c>
+      <c r="Y28">
         <v>1.5</v>
       </c>
-      <c r="Y28">
+      <c r="Z28">
         <v>34</v>
       </c>
-      <c r="AA28">
-        <v>4</v>
-      </c>
       <c r="AB28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>8</v>
       </c>
@@ -2742,23 +2751,23 @@
       <c r="U29">
         <v>18.5</v>
       </c>
-      <c r="V29">
+      <c r="W29">
         <v>10</v>
       </c>
-      <c r="X29">
-        <v>2</v>
-      </c>
       <c r="Y29">
+        <v>2</v>
+      </c>
+      <c r="Z29">
         <v>35</v>
       </c>
-      <c r="AA29">
+      <c r="AB29">
         <v>3.5</v>
       </c>
-      <c r="AB29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>8</v>
       </c>
@@ -2810,23 +2819,23 @@
       <c r="T30">
         <v>22</v>
       </c>
-      <c r="V30">
+      <c r="W30">
         <v>10</v>
       </c>
-      <c r="X30">
+      <c r="Y30">
         <v>2.5</v>
       </c>
-      <c r="Y30">
+      <c r="Z30">
         <v>34</v>
       </c>
-      <c r="AA30">
-        <v>4</v>
-      </c>
       <c r="AB30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>8</v>
       </c>
@@ -2878,23 +2887,23 @@
       <c r="T31">
         <v>22</v>
       </c>
-      <c r="V31">
+      <c r="W31">
         <v>10</v>
       </c>
-      <c r="X31">
-        <v>3</v>
-      </c>
       <c r="Y31">
+        <v>3</v>
+      </c>
+      <c r="Z31">
         <v>33</v>
       </c>
-      <c r="AA31">
-        <v>4</v>
-      </c>
       <c r="AB31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>9</v>
       </c>
@@ -2955,23 +2964,23 @@
       <c r="U32">
         <v>8.5</v>
       </c>
-      <c r="V32">
+      <c r="W32">
         <v>7.5</v>
       </c>
-      <c r="X32">
+      <c r="Y32">
         <v>1.5</v>
       </c>
-      <c r="Y32">
+      <c r="Z32">
         <v>33.5</v>
       </c>
-      <c r="AA32">
-        <v>4</v>
-      </c>
       <c r="AB32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>9</v>
       </c>
@@ -3032,23 +3041,23 @@
       <c r="U33">
         <v>8.5</v>
       </c>
-      <c r="V33">
+      <c r="W33">
         <v>8.5</v>
       </c>
-      <c r="X33">
+      <c r="Y33">
         <v>1.5</v>
       </c>
-      <c r="Z33">
+      <c r="AA33">
         <v>31</v>
       </c>
-      <c r="AA33">
+      <c r="AB33">
         <v>4.5</v>
       </c>
-      <c r="AB33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>9</v>
       </c>
@@ -3109,23 +3118,23 @@
       <c r="U34">
         <v>9.5</v>
       </c>
-      <c r="V34">
-        <v>8</v>
-      </c>
-      <c r="X34">
+      <c r="W34">
+        <v>8</v>
+      </c>
+      <c r="Y34">
         <v>1.5</v>
       </c>
-      <c r="Y34">
+      <c r="Z34">
         <v>34</v>
       </c>
-      <c r="AA34">
-        <v>4</v>
-      </c>
       <c r="AB34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>9</v>
       </c>
@@ -3186,23 +3195,23 @@
       <c r="U35">
         <v>9.5</v>
       </c>
-      <c r="V35">
+      <c r="W35">
         <v>8.5</v>
       </c>
-      <c r="X35">
+      <c r="Y35">
         <v>1.5</v>
       </c>
-      <c r="Z35">
+      <c r="AA35">
         <v>32</v>
       </c>
-      <c r="AA35">
+      <c r="AB35">
         <v>4.5</v>
       </c>
-      <c r="AB35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>9</v>
       </c>
@@ -3260,23 +3269,23 @@
       <c r="U36">
         <v>14.5</v>
       </c>
-      <c r="V36">
+      <c r="W36">
         <v>10</v>
       </c>
-      <c r="X36">
+      <c r="Y36">
         <v>1.5</v>
       </c>
-      <c r="Y36">
+      <c r="Z36">
         <v>35</v>
       </c>
-      <c r="AA36">
-        <v>4</v>
-      </c>
       <c r="AB36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>9</v>
       </c>
@@ -3334,23 +3343,23 @@
       <c r="T37">
         <v>17.5</v>
       </c>
-      <c r="V37">
-        <v>9</v>
-      </c>
-      <c r="X37">
+      <c r="W37">
+        <v>9</v>
+      </c>
+      <c r="Y37">
         <v>1.5</v>
       </c>
-      <c r="Y37">
+      <c r="Z37">
         <v>34</v>
       </c>
-      <c r="AA37">
-        <v>4</v>
-      </c>
       <c r="AB37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>9</v>
       </c>
@@ -3408,23 +3417,23 @@
       <c r="U38">
         <v>17.5</v>
       </c>
-      <c r="V38">
+      <c r="W38">
         <v>10</v>
       </c>
-      <c r="X38">
+      <c r="Y38">
         <v>1.5</v>
       </c>
-      <c r="Y38">
+      <c r="Z38">
         <v>36</v>
       </c>
-      <c r="AA38">
-        <v>4</v>
-      </c>
       <c r="AB38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>9</v>
       </c>
@@ -3482,23 +3491,23 @@
       <c r="T39">
         <v>19</v>
       </c>
-      <c r="V39">
-        <v>9</v>
-      </c>
-      <c r="X39">
+      <c r="W39">
+        <v>9</v>
+      </c>
+      <c r="Y39">
         <v>1.5</v>
       </c>
-      <c r="Y39">
+      <c r="Z39">
         <v>35.5</v>
       </c>
-      <c r="AA39">
-        <v>4</v>
-      </c>
       <c r="AB39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>10</v>
       </c>
@@ -3556,23 +3565,23 @@
       <c r="U40">
         <v>14</v>
       </c>
-      <c r="V40">
-        <v>9</v>
-      </c>
-      <c r="X40">
-        <v>2</v>
+      <c r="W40">
+        <v>9</v>
       </c>
       <c r="Y40">
+        <v>2</v>
+      </c>
+      <c r="Z40">
         <v>35</v>
       </c>
-      <c r="AA40">
-        <v>4</v>
-      </c>
       <c r="AB40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>10</v>
       </c>
@@ -3630,23 +3639,23 @@
       <c r="T41">
         <v>19</v>
       </c>
-      <c r="V41">
-        <v>8</v>
-      </c>
-      <c r="X41">
-        <v>2</v>
+      <c r="W41">
+        <v>8</v>
       </c>
       <c r="Y41">
+        <v>2</v>
+      </c>
+      <c r="Z41">
         <v>33</v>
       </c>
-      <c r="AA41">
-        <v>3</v>
-      </c>
       <c r="AB41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>10</v>
       </c>
@@ -3698,23 +3707,23 @@
       <c r="T42">
         <v>19</v>
       </c>
-      <c r="V42">
-        <v>9</v>
-      </c>
-      <c r="X42">
-        <v>2</v>
+      <c r="W42">
+        <v>9</v>
       </c>
       <c r="Y42">
+        <v>2</v>
+      </c>
+      <c r="Z42">
         <v>34</v>
       </c>
-      <c r="AA42">
-        <v>3</v>
-      </c>
       <c r="AB42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>11</v>
       </c>
@@ -3775,23 +3784,23 @@
       <c r="U43">
         <v>8</v>
       </c>
-      <c r="V43">
-        <v>8</v>
-      </c>
-      <c r="X43">
-        <v>2</v>
+      <c r="W43">
+        <v>8</v>
       </c>
       <c r="Y43">
+        <v>2</v>
+      </c>
+      <c r="Z43">
         <v>36</v>
       </c>
-      <c r="AA43">
-        <v>4</v>
-      </c>
       <c r="AB43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>11</v>
       </c>
@@ -3849,23 +3858,23 @@
       <c r="T44">
         <v>19</v>
       </c>
-      <c r="V44">
-        <v>9</v>
-      </c>
-      <c r="X44">
-        <v>2</v>
+      <c r="W44">
+        <v>9</v>
       </c>
       <c r="Y44">
+        <v>2</v>
+      </c>
+      <c r="Z44">
         <v>36</v>
       </c>
-      <c r="AA44">
-        <v>4</v>
-      </c>
       <c r="AB44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>11</v>
       </c>
@@ -3923,23 +3932,23 @@
       <c r="U45">
         <v>15</v>
       </c>
-      <c r="V45">
+      <c r="W45">
         <v>11</v>
       </c>
-      <c r="X45">
-        <v>2</v>
-      </c>
       <c r="Y45">
+        <v>2</v>
+      </c>
+      <c r="Z45">
         <v>37</v>
       </c>
-      <c r="AA45">
+      <c r="AB45">
         <v>4.5</v>
       </c>
-      <c r="AB45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>11</v>
       </c>
@@ -3997,23 +4006,23 @@
       <c r="T46">
         <v>20</v>
       </c>
-      <c r="V46">
+      <c r="W46">
         <v>11</v>
       </c>
-      <c r="X46">
-        <v>2</v>
-      </c>
-      <c r="Z46">
+      <c r="Y46">
+        <v>2</v>
+      </c>
+      <c r="AA46">
         <v>32</v>
       </c>
-      <c r="AA46">
+      <c r="AB46">
         <v>6</v>
       </c>
-      <c r="AB46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>11</v>
       </c>
@@ -4071,23 +4080,23 @@
       <c r="U47">
         <v>15</v>
       </c>
-      <c r="V47">
+      <c r="W47">
         <v>14</v>
       </c>
-      <c r="X47">
-        <v>3</v>
-      </c>
-      <c r="Z47">
+      <c r="Y47">
+        <v>3</v>
+      </c>
+      <c r="AA47">
         <v>32</v>
       </c>
-      <c r="AA47">
+      <c r="AB47">
         <v>5</v>
       </c>
-      <c r="AB47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>11</v>
       </c>
@@ -4139,23 +4148,23 @@
       <c r="T48">
         <v>21</v>
       </c>
-      <c r="V48">
+      <c r="W48">
         <v>10</v>
       </c>
-      <c r="X48">
-        <v>3</v>
-      </c>
       <c r="Y48">
+        <v>3</v>
+      </c>
+      <c r="Z48">
         <v>37</v>
       </c>
-      <c r="AA48">
+      <c r="AB48">
         <v>3.5</v>
       </c>
-      <c r="AB48">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>11</v>
       </c>
@@ -4207,23 +4216,23 @@
       <c r="T49">
         <v>20</v>
       </c>
-      <c r="V49">
+      <c r="W49">
         <v>11</v>
       </c>
-      <c r="X49">
+      <c r="Y49">
         <v>2.5</v>
       </c>
-      <c r="Y49">
+      <c r="Z49">
         <v>36</v>
       </c>
-      <c r="AA49">
-        <v>4</v>
-      </c>
       <c r="AB49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>12</v>
       </c>
@@ -4281,23 +4290,23 @@
       <c r="T50">
         <v>19</v>
       </c>
-      <c r="V50">
-        <v>8</v>
-      </c>
-      <c r="X50">
-        <v>2</v>
-      </c>
-      <c r="Z50">
+      <c r="W50">
+        <v>8</v>
+      </c>
+      <c r="Y50">
+        <v>2</v>
+      </c>
+      <c r="AA50">
         <v>36</v>
       </c>
-      <c r="AA50">
-        <v>4</v>
-      </c>
       <c r="AB50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>12</v>
       </c>
@@ -4355,23 +4364,23 @@
       <c r="U51">
         <v>15</v>
       </c>
-      <c r="V51">
+      <c r="W51">
         <v>10</v>
       </c>
-      <c r="X51">
-        <v>2</v>
-      </c>
-      <c r="Z51">
+      <c r="Y51">
+        <v>2</v>
+      </c>
+      <c r="AA51">
         <v>36</v>
       </c>
-      <c r="AA51">
+      <c r="AB51">
         <v>3.5</v>
       </c>
-      <c r="AB51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>13</v>
       </c>
@@ -4432,23 +4441,23 @@
       <c r="U52">
         <v>8</v>
       </c>
-      <c r="V52">
+      <c r="W52">
         <v>7</v>
       </c>
-      <c r="X52">
-        <v>1</v>
-      </c>
-      <c r="Z52">
+      <c r="Y52">
+        <v>1</v>
+      </c>
+      <c r="AA52">
         <v>35</v>
       </c>
-      <c r="AA52">
-        <v>4</v>
-      </c>
       <c r="AB52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>13</v>
       </c>
@@ -4506,23 +4515,23 @@
       <c r="T53">
         <v>20</v>
       </c>
-      <c r="V53">
-        <v>8</v>
-      </c>
-      <c r="X53">
-        <v>1</v>
-      </c>
-      <c r="Z53">
+      <c r="W53">
+        <v>8</v>
+      </c>
+      <c r="Y53">
+        <v>1</v>
+      </c>
+      <c r="AA53">
         <v>34</v>
       </c>
-      <c r="AA53">
-        <v>4</v>
-      </c>
       <c r="AB53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>13</v>
       </c>
@@ -4580,23 +4589,23 @@
       <c r="U54">
         <v>16</v>
       </c>
-      <c r="V54">
-        <v>9</v>
-      </c>
-      <c r="X54">
-        <v>1</v>
-      </c>
-      <c r="Z54">
+      <c r="W54">
+        <v>9</v>
+      </c>
+      <c r="Y54">
+        <v>1</v>
+      </c>
+      <c r="AA54">
         <v>36</v>
       </c>
-      <c r="AA54">
-        <v>4</v>
-      </c>
       <c r="AB54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>13</v>
       </c>
@@ -4654,23 +4663,23 @@
       <c r="T55">
         <v>20</v>
       </c>
-      <c r="V55">
-        <v>8</v>
-      </c>
-      <c r="X55">
-        <v>1</v>
-      </c>
-      <c r="Z55">
+      <c r="W55">
+        <v>8</v>
+      </c>
+      <c r="Y55">
+        <v>1</v>
+      </c>
+      <c r="AA55">
         <v>35</v>
       </c>
-      <c r="AA55">
-        <v>4</v>
-      </c>
       <c r="AB55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>13</v>
       </c>
@@ -4728,23 +4737,23 @@
       <c r="U56">
         <v>16</v>
       </c>
-      <c r="V56">
-        <v>8</v>
-      </c>
-      <c r="X56">
-        <v>2</v>
-      </c>
-      <c r="Z56">
+      <c r="W56">
+        <v>8</v>
+      </c>
+      <c r="Y56">
+        <v>2</v>
+      </c>
+      <c r="AA56">
         <v>36</v>
       </c>
-      <c r="AA56">
+      <c r="AB56">
         <v>5</v>
       </c>
-      <c r="AB56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>14</v>
       </c>
@@ -4805,20 +4814,20 @@
       <c r="U57">
         <v>7</v>
       </c>
-      <c r="V57">
-        <v>8</v>
-      </c>
-      <c r="Z57">
+      <c r="W57">
+        <v>8</v>
+      </c>
+      <c r="AA57">
         <v>35</v>
       </c>
-      <c r="AA57">
-        <v>3</v>
-      </c>
       <c r="AB57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>14</v>
       </c>
@@ -4876,20 +4885,20 @@
       <c r="U58">
         <v>16</v>
       </c>
-      <c r="V58">
-        <v>12</v>
-      </c>
-      <c r="Z58">
+      <c r="W58">
+        <v>12</v>
+      </c>
+      <c r="AA58">
         <v>36</v>
       </c>
-      <c r="AA58">
-        <v>3</v>
-      </c>
       <c r="AB58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>14</v>
       </c>
@@ -4947,20 +4956,20 @@
       <c r="T59">
         <v>22</v>
       </c>
-      <c r="V59">
-        <v>9</v>
-      </c>
-      <c r="Z59">
+      <c r="W59">
+        <v>9</v>
+      </c>
+      <c r="AA59">
         <v>34</v>
       </c>
-      <c r="AA59">
-        <v>4</v>
-      </c>
       <c r="AB59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>15</v>
       </c>
@@ -5015,20 +5024,20 @@
       <c r="U60">
         <v>8</v>
       </c>
-      <c r="V60">
+      <c r="W60">
         <v>7</v>
       </c>
-      <c r="Z60">
+      <c r="AA60">
         <v>37</v>
       </c>
-      <c r="AA60">
-        <v>3</v>
-      </c>
       <c r="AB60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>16</v>
       </c>
@@ -5086,26 +5095,26 @@
       <c r="T61">
         <v>16.5</v>
       </c>
-      <c r="V61">
-        <v>8</v>
-      </c>
       <c r="W61">
+        <v>8</v>
+      </c>
+      <c r="X61">
         <v>2.5</v>
       </c>
-      <c r="X61">
+      <c r="Y61">
         <v>1.5</v>
       </c>
-      <c r="Z61">
+      <c r="AA61">
         <v>35</v>
       </c>
-      <c r="AA61">
-        <v>3</v>
-      </c>
       <c r="AB61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>16</v>
       </c>
@@ -5163,26 +5172,26 @@
       <c r="U62">
         <v>13.5</v>
       </c>
-      <c r="V62">
+      <c r="W62">
         <v>11</v>
       </c>
-      <c r="W62">
+      <c r="X62">
         <v>3.5</v>
       </c>
-      <c r="X62">
+      <c r="Y62">
         <v>1.5</v>
       </c>
-      <c r="Z62">
+      <c r="AA62">
         <v>34</v>
       </c>
-      <c r="AA62">
+      <c r="AB62">
         <v>3.5</v>
       </c>
-      <c r="AB62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>16</v>
       </c>
@@ -5243,23 +5252,23 @@
       <c r="U63">
         <v>7.5</v>
       </c>
-      <c r="V63">
+      <c r="W63">
         <v>8.5</v>
       </c>
-      <c r="X63">
+      <c r="Y63">
         <v>1.5</v>
       </c>
-      <c r="Z63">
+      <c r="AA63">
         <v>35</v>
       </c>
-      <c r="AA63">
-        <v>3</v>
-      </c>
       <c r="AB63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>16</v>
       </c>
@@ -5317,26 +5326,26 @@
       <c r="T64">
         <v>18</v>
       </c>
-      <c r="V64">
-        <v>8</v>
-      </c>
       <c r="W64">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="X64">
+        <v>3</v>
+      </c>
+      <c r="Y64">
         <v>1.5</v>
       </c>
-      <c r="Z64">
+      <c r="AA64">
         <v>34.5</v>
       </c>
-      <c r="AA64">
-        <v>3</v>
-      </c>
       <c r="AB64">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>17</v>
       </c>
@@ -5394,23 +5403,23 @@
       <c r="T65">
         <v>17</v>
       </c>
-      <c r="V65">
+      <c r="W65">
         <v>7</v>
       </c>
-      <c r="X65">
-        <v>3</v>
-      </c>
-      <c r="Z65">
+      <c r="Y65">
+        <v>3</v>
+      </c>
+      <c r="AA65">
         <v>35</v>
       </c>
-      <c r="AA65">
-        <v>4</v>
-      </c>
       <c r="AB65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>17</v>
       </c>
@@ -5468,23 +5477,23 @@
       <c r="U66">
         <v>15</v>
       </c>
-      <c r="V66">
-        <v>9</v>
-      </c>
-      <c r="X66">
-        <v>2</v>
-      </c>
-      <c r="Z66">
+      <c r="W66">
+        <v>9</v>
+      </c>
+      <c r="Y66">
+        <v>2</v>
+      </c>
+      <c r="AA66">
         <v>37</v>
       </c>
-      <c r="AA66">
-        <v>3</v>
-      </c>
       <c r="AB66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>17</v>
       </c>
@@ -5542,23 +5551,23 @@
       <c r="T67">
         <v>19</v>
       </c>
-      <c r="V67">
+      <c r="W67">
         <v>7</v>
       </c>
-      <c r="X67">
-        <v>2</v>
-      </c>
-      <c r="Z67">
+      <c r="Y67">
+        <v>2</v>
+      </c>
+      <c r="AA67">
         <v>35</v>
       </c>
-      <c r="AA67">
-        <v>4</v>
-      </c>
       <c r="AB67">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>17</v>
       </c>
@@ -5616,23 +5625,23 @@
       <c r="U68">
         <v>14</v>
       </c>
-      <c r="V68">
-        <v>9</v>
-      </c>
-      <c r="X68">
-        <v>2</v>
-      </c>
-      <c r="Z68">
+      <c r="W68">
+        <v>9</v>
+      </c>
+      <c r="Y68">
+        <v>2</v>
+      </c>
+      <c r="AA68">
         <v>38</v>
       </c>
-      <c r="AA68">
-        <v>4</v>
-      </c>
       <c r="AB68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>18</v>
       </c>
@@ -5690,23 +5699,23 @@
       <c r="T69">
         <v>18</v>
       </c>
-      <c r="V69">
-        <v>8</v>
-      </c>
-      <c r="X69">
+      <c r="W69">
+        <v>8</v>
+      </c>
+      <c r="Y69">
         <v>1.5</v>
       </c>
-      <c r="Z69">
+      <c r="AA69">
         <v>33</v>
       </c>
-      <c r="AA69">
+      <c r="AB69">
         <v>3.5</v>
       </c>
-      <c r="AB69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>18</v>
       </c>
@@ -5764,23 +5773,23 @@
       <c r="U70">
         <v>14</v>
       </c>
-      <c r="V70">
-        <v>9</v>
-      </c>
-      <c r="X70">
+      <c r="W70">
+        <v>9</v>
+      </c>
+      <c r="Y70">
         <v>1.5</v>
       </c>
-      <c r="Z70">
+      <c r="AA70">
         <v>34</v>
       </c>
-      <c r="AA70">
-        <v>3</v>
-      </c>
       <c r="AB70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>18</v>
       </c>
@@ -5832,23 +5841,23 @@
       <c r="T71">
         <v>19</v>
       </c>
-      <c r="V71">
-        <v>8</v>
-      </c>
-      <c r="X71">
+      <c r="W71">
+        <v>8</v>
+      </c>
+      <c r="Y71">
         <v>2.5</v>
       </c>
-      <c r="Z71">
+      <c r="AA71">
         <v>33</v>
       </c>
-      <c r="AA71">
+      <c r="AB71">
         <v>3.5</v>
       </c>
-      <c r="AB71">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>18</v>
       </c>
@@ -5900,23 +5909,23 @@
       <c r="U72">
         <v>15</v>
       </c>
-      <c r="V72">
-        <v>9</v>
-      </c>
-      <c r="X72">
-        <v>2</v>
-      </c>
-      <c r="Z72">
+      <c r="W72">
+        <v>9</v>
+      </c>
+      <c r="Y72">
+        <v>2</v>
+      </c>
+      <c r="AA72">
         <v>34</v>
       </c>
-      <c r="AA72">
-        <v>3</v>
-      </c>
       <c r="AB72">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>18</v>
       </c>
@@ -5968,23 +5977,23 @@
       <c r="T73">
         <v>21</v>
       </c>
-      <c r="V73">
-        <v>8</v>
-      </c>
-      <c r="X73">
-        <v>2</v>
-      </c>
-      <c r="Z73">
+      <c r="W73">
+        <v>8</v>
+      </c>
+      <c r="Y73">
+        <v>2</v>
+      </c>
+      <c r="AA73">
         <v>34</v>
       </c>
-      <c r="AA73">
+      <c r="AB73">
         <v>2.5</v>
       </c>
-      <c r="AB73">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>19</v>
       </c>
@@ -6042,26 +6051,26 @@
       <c r="T74">
         <v>17</v>
       </c>
-      <c r="V74">
+      <c r="W74">
         <v>6.5</v>
       </c>
-      <c r="W74">
-        <v>2</v>
-      </c>
       <c r="X74">
-        <v>3</v>
-      </c>
-      <c r="Z74">
+        <v>2</v>
+      </c>
+      <c r="Y74">
+        <v>3</v>
+      </c>
+      <c r="AA74">
         <v>34</v>
       </c>
-      <c r="AA74">
-        <v>4</v>
-      </c>
       <c r="AB74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>19</v>
       </c>
@@ -6119,26 +6128,26 @@
       <c r="U75">
         <v>12</v>
       </c>
-      <c r="V75">
+      <c r="W75">
         <v>9.5</v>
       </c>
-      <c r="W75">
+      <c r="X75">
         <v>2.5</v>
       </c>
-      <c r="X75">
-        <v>2</v>
-      </c>
-      <c r="Z75">
+      <c r="Y75">
+        <v>2</v>
+      </c>
+      <c r="AA75">
         <v>34.5</v>
       </c>
-      <c r="AA75">
-        <v>4</v>
-      </c>
       <c r="AB75">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>20</v>
       </c>
@@ -6196,26 +6205,26 @@
       <c r="T76">
         <v>18.100000000000001</v>
       </c>
-      <c r="V76">
+      <c r="W76">
         <v>7.8</v>
       </c>
-      <c r="W76">
+      <c r="X76">
         <v>2.9</v>
       </c>
-      <c r="X76">
+      <c r="Y76">
         <v>3.2</v>
       </c>
-      <c r="Z76">
+      <c r="AA76">
         <v>30.1</v>
       </c>
-      <c r="AA76">
+      <c r="AB76">
         <v>3.8</v>
       </c>
-      <c r="AB76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>20</v>
       </c>
@@ -6273,26 +6282,26 @@
       <c r="U77">
         <v>13.8</v>
       </c>
-      <c r="V77">
+      <c r="W77">
         <v>9.6999999999999993</v>
       </c>
-      <c r="W77">
+      <c r="X77">
         <v>3.9</v>
       </c>
-      <c r="X77">
-        <v>4</v>
-      </c>
-      <c r="Z77">
+      <c r="Y77">
+        <v>4</v>
+      </c>
+      <c r="AA77">
         <v>29.9</v>
       </c>
-      <c r="AA77">
+      <c r="AB77">
         <v>4.2</v>
       </c>
-      <c r="AB77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>21</v>
       </c>
@@ -6350,23 +6359,23 @@
       <c r="T78">
         <v>19</v>
       </c>
-      <c r="V78">
+      <c r="W78">
         <v>7.5</v>
       </c>
-      <c r="X78">
-        <v>2</v>
-      </c>
-      <c r="Z78">
+      <c r="Y78">
+        <v>2</v>
+      </c>
+      <c r="AA78">
         <v>34.5</v>
       </c>
-      <c r="AA78">
-        <v>3</v>
-      </c>
       <c r="AB78">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>21</v>
       </c>
@@ -6424,23 +6433,23 @@
       <c r="U79">
         <v>14</v>
       </c>
-      <c r="V79">
+      <c r="W79">
         <v>9.5</v>
       </c>
-      <c r="X79">
+      <c r="Y79">
         <v>2.5</v>
       </c>
-      <c r="Z79">
+      <c r="AA79">
         <v>35</v>
       </c>
-      <c r="AA79">
-        <v>3</v>
-      </c>
       <c r="AB79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>22</v>
       </c>
@@ -6498,26 +6507,26 @@
       <c r="T80">
         <v>18.2</v>
       </c>
-      <c r="V80">
+      <c r="W80">
         <v>7.5</v>
       </c>
-      <c r="W80">
+      <c r="X80">
         <v>3.2</v>
       </c>
-      <c r="X80">
+      <c r="Y80">
         <v>2.9</v>
       </c>
-      <c r="Z80">
+      <c r="AA80">
         <v>30</v>
       </c>
-      <c r="AA80">
+      <c r="AB80">
         <v>3.5</v>
       </c>
-      <c r="AB80">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>22</v>
       </c>
@@ -6575,26 +6584,26 @@
       <c r="U81">
         <v>13.5</v>
       </c>
-      <c r="V81">
+      <c r="W81">
         <v>8.9</v>
       </c>
-      <c r="W81">
-        <v>4</v>
-      </c>
       <c r="X81">
+        <v>4</v>
+      </c>
+      <c r="Y81">
         <v>2.8</v>
       </c>
-      <c r="Z81">
+      <c r="AA81">
         <v>31.6</v>
       </c>
-      <c r="AA81">
-        <v>4</v>
-      </c>
       <c r="AB81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>23</v>
       </c>
@@ -6652,20 +6661,20 @@
       <c r="T82">
         <v>20</v>
       </c>
-      <c r="V82">
-        <v>8</v>
-      </c>
-      <c r="Z82">
+      <c r="W82">
+        <v>8</v>
+      </c>
+      <c r="AA82">
         <v>33</v>
       </c>
-      <c r="AA82">
-        <v>3</v>
-      </c>
       <c r="AB82">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>23</v>
       </c>
@@ -6723,20 +6732,20 @@
       <c r="U83">
         <v>13</v>
       </c>
-      <c r="V83">
+      <c r="W83">
         <v>11</v>
       </c>
-      <c r="Z83">
+      <c r="AA83">
         <v>35</v>
       </c>
-      <c r="AA83">
-        <v>3</v>
-      </c>
       <c r="AB83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:28" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="AC83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>24</v>
       </c>
@@ -6794,23 +6803,23 @@
       <c r="U84">
         <v>14</v>
       </c>
-      <c r="V84">
-        <v>12</v>
-      </c>
-      <c r="X84">
-        <v>2</v>
-      </c>
-      <c r="Z84">
+      <c r="W84">
+        <v>12</v>
+      </c>
+      <c r="Y84">
+        <v>2</v>
+      </c>
+      <c r="AA84">
         <v>34</v>
       </c>
-      <c r="AA84">
-        <v>4</v>
-      </c>
       <c r="AB84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>24</v>
       </c>
@@ -6868,23 +6877,23 @@
       <c r="T85">
         <v>19</v>
       </c>
-      <c r="V85">
+      <c r="W85">
         <v>10</v>
       </c>
-      <c r="X85">
-        <v>3</v>
-      </c>
-      <c r="Z85">
+      <c r="Y85">
+        <v>3</v>
+      </c>
+      <c r="AA85">
         <v>34</v>
       </c>
-      <c r="AA85">
-        <v>4</v>
-      </c>
       <c r="AB85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>25</v>
       </c>
@@ -6942,23 +6951,23 @@
       <c r="T86">
         <v>17.5</v>
       </c>
-      <c r="V86">
-        <v>8</v>
-      </c>
-      <c r="X86">
-        <v>2</v>
-      </c>
-      <c r="Z86">
+      <c r="W86">
+        <v>8</v>
+      </c>
+      <c r="Y86">
+        <v>2</v>
+      </c>
+      <c r="AA86">
         <v>33.5</v>
       </c>
-      <c r="AA86">
-        <v>4</v>
-      </c>
       <c r="AB86">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>25</v>
       </c>
@@ -7016,23 +7025,23 @@
       <c r="U87">
         <v>13</v>
       </c>
-      <c r="V87">
+      <c r="W87">
         <v>10</v>
       </c>
-      <c r="X87">
-        <v>2</v>
-      </c>
-      <c r="Z87">
+      <c r="Y87">
+        <v>2</v>
+      </c>
+      <c r="AA87">
         <v>34</v>
       </c>
-      <c r="AA87">
+      <c r="AB87">
         <v>4.5</v>
       </c>
-      <c r="AB87">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>26</v>
       </c>
@@ -7090,23 +7099,23 @@
       <c r="T88">
         <v>17</v>
       </c>
-      <c r="V88">
+      <c r="W88">
         <v>7</v>
       </c>
-      <c r="X88">
-        <v>3</v>
-      </c>
-      <c r="Z88">
+      <c r="Y88">
+        <v>3</v>
+      </c>
+      <c r="AA88">
         <v>34</v>
       </c>
-      <c r="AA88">
+      <c r="AB88">
         <v>5</v>
       </c>
-      <c r="AB88">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>26</v>
       </c>
@@ -7164,23 +7173,23 @@
       <c r="U89">
         <v>14</v>
       </c>
-      <c r="V89">
-        <v>9</v>
-      </c>
-      <c r="X89">
-        <v>2</v>
-      </c>
-      <c r="Z89">
+      <c r="W89">
+        <v>9</v>
+      </c>
+      <c r="Y89">
+        <v>2</v>
+      </c>
+      <c r="AA89">
         <v>35</v>
       </c>
-      <c r="AA89">
+      <c r="AB89">
         <v>5</v>
       </c>
-      <c r="AB89">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>26</v>
       </c>
@@ -7238,23 +7247,23 @@
       <c r="T90">
         <v>19</v>
       </c>
-      <c r="V90">
-        <v>9</v>
-      </c>
-      <c r="X90">
-        <v>2</v>
-      </c>
-      <c r="Z90">
+      <c r="W90">
+        <v>9</v>
+      </c>
+      <c r="Y90">
+        <v>2</v>
+      </c>
+      <c r="AA90">
         <v>33</v>
       </c>
-      <c r="AA90">
+      <c r="AB90">
         <v>5</v>
       </c>
-      <c r="AB90">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>26</v>
       </c>
@@ -7312,23 +7321,23 @@
       <c r="U91">
         <v>15</v>
       </c>
-      <c r="V91">
+      <c r="W91">
         <v>10</v>
       </c>
-      <c r="X91">
-        <v>2</v>
-      </c>
-      <c r="Z91">
+      <c r="Y91">
+        <v>2</v>
+      </c>
+      <c r="AA91">
         <v>36</v>
       </c>
-      <c r="AA91">
+      <c r="AB91">
         <v>5</v>
       </c>
-      <c r="AB91">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>27</v>
       </c>
@@ -7386,23 +7395,23 @@
       <c r="T92">
         <v>18.8</v>
       </c>
-      <c r="V92">
+      <c r="W92">
         <v>7.6</v>
       </c>
-      <c r="X92">
+      <c r="Y92">
         <v>3.2</v>
       </c>
-      <c r="Z92">
+      <c r="AA92">
         <v>30.8</v>
       </c>
-      <c r="AA92">
+      <c r="AB92">
         <v>3.5</v>
       </c>
-      <c r="AB92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>27</v>
       </c>
@@ -7460,23 +7469,23 @@
       <c r="U93">
         <v>13.4</v>
       </c>
-      <c r="V93">
+      <c r="W93">
         <v>9.5</v>
       </c>
-      <c r="X93">
+      <c r="Y93">
         <v>3.2</v>
       </c>
-      <c r="Z93">
+      <c r="AA93">
         <v>31</v>
       </c>
-      <c r="AA93">
+      <c r="AB93">
         <v>3.6</v>
       </c>
-      <c r="AB93">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>27</v>
       </c>
@@ -7534,20 +7543,20 @@
       <c r="T94">
         <v>19.399999999999999</v>
       </c>
-      <c r="V94">
+      <c r="W94">
         <v>7.6</v>
       </c>
-      <c r="X94">
-        <v>4</v>
-      </c>
-      <c r="Z94">
+      <c r="Y94">
+        <v>4</v>
+      </c>
+      <c r="AA94">
         <v>30.2</v>
       </c>
-      <c r="AB94">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>28</v>
       </c>
@@ -7605,23 +7614,23 @@
       <c r="T95">
         <v>16</v>
       </c>
-      <c r="V95">
-        <v>8</v>
-      </c>
-      <c r="X95">
-        <v>2</v>
-      </c>
-      <c r="Z95">
+      <c r="W95">
+        <v>8</v>
+      </c>
+      <c r="Y95">
+        <v>2</v>
+      </c>
+      <c r="AA95">
         <v>35</v>
       </c>
-      <c r="AA95">
+      <c r="AB95">
         <v>5</v>
       </c>
-      <c r="AB95">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>28</v>
       </c>
@@ -7679,23 +7688,23 @@
       <c r="U96">
         <v>12</v>
       </c>
-      <c r="V96">
+      <c r="W96">
         <v>10</v>
       </c>
-      <c r="X96">
-        <v>2</v>
-      </c>
-      <c r="Z96">
+      <c r="Y96">
+        <v>2</v>
+      </c>
+      <c r="AA96">
         <v>36</v>
       </c>
-      <c r="AA96">
+      <c r="AB96">
         <v>6</v>
       </c>
-      <c r="AB96">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>28</v>
       </c>
@@ -7753,23 +7762,23 @@
       <c r="T97">
         <v>16</v>
       </c>
-      <c r="V97">
-        <v>9</v>
-      </c>
-      <c r="X97">
-        <v>2</v>
-      </c>
-      <c r="Z97">
+      <c r="W97">
+        <v>9</v>
+      </c>
+      <c r="Y97">
+        <v>2</v>
+      </c>
+      <c r="AA97">
         <v>35</v>
       </c>
-      <c r="AA97">
+      <c r="AB97">
         <v>5</v>
       </c>
-      <c r="AB97">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>28</v>
       </c>
@@ -7827,23 +7836,23 @@
       <c r="U98">
         <v>13</v>
       </c>
-      <c r="V98">
+      <c r="W98">
         <v>10</v>
       </c>
-      <c r="X98">
-        <v>2</v>
-      </c>
-      <c r="Z98">
+      <c r="Y98">
+        <v>2</v>
+      </c>
+      <c r="AA98">
         <v>36</v>
       </c>
-      <c r="AA98">
+      <c r="AB98">
         <v>5</v>
       </c>
-      <c r="AB98">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>29</v>
       </c>
@@ -7901,23 +7910,23 @@
       <c r="T99">
         <v>17</v>
       </c>
-      <c r="V99">
+      <c r="W99">
         <v>7</v>
       </c>
-      <c r="X99">
-        <v>2</v>
-      </c>
-      <c r="Z99">
+      <c r="Y99">
+        <v>2</v>
+      </c>
+      <c r="AA99">
         <v>36</v>
       </c>
-      <c r="AA99">
-        <v>4</v>
-      </c>
       <c r="AB99">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>29</v>
       </c>
@@ -7975,23 +7984,23 @@
       <c r="U100">
         <v>12</v>
       </c>
-      <c r="V100">
+      <c r="W100">
         <v>10</v>
       </c>
-      <c r="X100">
-        <v>2</v>
-      </c>
-      <c r="Z100">
+      <c r="Y100">
+        <v>2</v>
+      </c>
+      <c r="AA100">
         <v>36</v>
       </c>
-      <c r="AA100">
+      <c r="AB100">
         <v>5</v>
       </c>
-      <c r="AB100">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>29</v>
       </c>
@@ -8049,23 +8058,23 @@
       <c r="T101">
         <v>17</v>
       </c>
-      <c r="V101">
-        <v>8</v>
-      </c>
-      <c r="X101">
-        <v>2</v>
-      </c>
-      <c r="Z101">
+      <c r="W101">
+        <v>8</v>
+      </c>
+      <c r="Y101">
+        <v>2</v>
+      </c>
+      <c r="AA101">
         <v>36</v>
       </c>
-      <c r="AA101">
-        <v>4</v>
-      </c>
       <c r="AB101">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>29</v>
       </c>
@@ -8123,23 +8132,23 @@
       <c r="U102">
         <v>12</v>
       </c>
-      <c r="V102">
+      <c r="W102">
         <v>10</v>
       </c>
-      <c r="X102">
-        <v>2</v>
-      </c>
-      <c r="Z102">
+      <c r="Y102">
+        <v>2</v>
+      </c>
+      <c r="AA102">
         <v>37</v>
       </c>
-      <c r="AA102">
+      <c r="AB102">
         <v>5</v>
       </c>
-      <c r="AB102">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>30</v>
       </c>
@@ -8197,23 +8206,23 @@
       <c r="U103">
         <v>11</v>
       </c>
-      <c r="V103">
-        <v>9</v>
-      </c>
-      <c r="X103">
-        <v>2</v>
-      </c>
-      <c r="Z103">
+      <c r="W103">
+        <v>9</v>
+      </c>
+      <c r="Y103">
+        <v>2</v>
+      </c>
+      <c r="AA103">
         <v>37</v>
       </c>
-      <c r="AA103">
-        <v>4</v>
-      </c>
       <c r="AB103">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>30</v>
       </c>
@@ -8271,23 +8280,23 @@
       <c r="T104">
         <v>15</v>
       </c>
-      <c r="V104">
-        <v>8</v>
-      </c>
-      <c r="X104">
-        <v>2</v>
-      </c>
-      <c r="Z104">
+      <c r="W104">
+        <v>8</v>
+      </c>
+      <c r="Y104">
+        <v>2</v>
+      </c>
+      <c r="AA104">
         <v>35</v>
       </c>
-      <c r="AA104">
-        <v>4</v>
-      </c>
       <c r="AB104">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:28" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="AC104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>31</v>
       </c>
@@ -8345,23 +8354,23 @@
       <c r="T105">
         <v>17</v>
       </c>
-      <c r="V105">
+      <c r="W105">
         <v>6.5</v>
       </c>
-      <c r="X105">
-        <v>2</v>
-      </c>
-      <c r="Z105">
+      <c r="Y105">
+        <v>2</v>
+      </c>
+      <c r="AA105">
         <v>37</v>
       </c>
-      <c r="AA105">
+      <c r="AB105">
         <v>4.5</v>
       </c>
-      <c r="AB105">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>31</v>
       </c>
@@ -8419,19 +8428,546 @@
       <c r="U106">
         <v>11</v>
       </c>
-      <c r="V106">
-        <v>9</v>
-      </c>
-      <c r="X106">
-        <v>2</v>
-      </c>
-      <c r="Z106">
+      <c r="W106">
+        <v>9</v>
+      </c>
+      <c r="Y106">
+        <v>2</v>
+      </c>
+      <c r="AA106">
         <v>38</v>
       </c>
-      <c r="AA106">
+      <c r="AB106">
         <v>4.5</v>
       </c>
-      <c r="AB106">
+      <c r="AC106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <v>32</v>
+      </c>
+      <c r="B107">
+        <v>2026</v>
+      </c>
+      <c r="C107">
+        <v>10</v>
+      </c>
+      <c r="D107">
+        <v>12</v>
+      </c>
+      <c r="E107">
+        <v>10</v>
+      </c>
+      <c r="F107">
+        <v>14</v>
+      </c>
+      <c r="G107" t="s">
+        <v>11</v>
+      </c>
+      <c r="H107" t="s">
+        <v>13</v>
+      </c>
+      <c r="I107" t="s">
+        <v>12</v>
+      </c>
+      <c r="J107">
+        <v>834</v>
+      </c>
+      <c r="K107">
+        <v>0</v>
+      </c>
+      <c r="L107">
+        <v>1</v>
+      </c>
+      <c r="M107">
+        <v>0.5</v>
+      </c>
+      <c r="N107">
+        <v>0.5</v>
+      </c>
+      <c r="O107">
+        <v>16</v>
+      </c>
+      <c r="P107">
+        <v>3</v>
+      </c>
+      <c r="Q107">
+        <v>13.5</v>
+      </c>
+      <c r="S107">
+        <v>2.5</v>
+      </c>
+      <c r="T107">
+        <v>18</v>
+      </c>
+      <c r="W107">
+        <v>6.5</v>
+      </c>
+      <c r="Y107">
+        <v>2</v>
+      </c>
+      <c r="AA107">
+        <v>35</v>
+      </c>
+      <c r="AB107">
+        <v>3</v>
+      </c>
+      <c r="AC107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <v>32</v>
+      </c>
+      <c r="B108">
+        <v>2026</v>
+      </c>
+      <c r="C108">
+        <v>10</v>
+      </c>
+      <c r="D108">
+        <v>12</v>
+      </c>
+      <c r="E108">
+        <v>10</v>
+      </c>
+      <c r="F108">
+        <v>14</v>
+      </c>
+      <c r="G108" t="s">
+        <v>11</v>
+      </c>
+      <c r="H108" t="s">
+        <v>13</v>
+      </c>
+      <c r="I108" t="s">
+        <v>12</v>
+      </c>
+      <c r="J108">
+        <v>815</v>
+      </c>
+      <c r="K108">
+        <v>0</v>
+      </c>
+      <c r="L108">
+        <v>1</v>
+      </c>
+      <c r="M108">
+        <v>0.5</v>
+      </c>
+      <c r="N108">
+        <v>0.5</v>
+      </c>
+      <c r="O108">
+        <v>17</v>
+      </c>
+      <c r="P108">
+        <v>2.5</v>
+      </c>
+      <c r="Q108">
+        <v>16</v>
+      </c>
+      <c r="S108">
+        <v>2</v>
+      </c>
+      <c r="U108">
+        <v>13</v>
+      </c>
+      <c r="W108">
+        <v>8</v>
+      </c>
+      <c r="Y108">
+        <v>2</v>
+      </c>
+      <c r="AA108">
+        <v>36</v>
+      </c>
+      <c r="AB108">
+        <v>3</v>
+      </c>
+      <c r="AC108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <v>33</v>
+      </c>
+      <c r="B109">
+        <v>2026</v>
+      </c>
+      <c r="C109">
+        <v>10</v>
+      </c>
+      <c r="D109">
+        <v>14</v>
+      </c>
+      <c r="E109">
+        <v>10</v>
+      </c>
+      <c r="F109">
+        <v>16</v>
+      </c>
+      <c r="G109" t="s">
+        <v>29</v>
+      </c>
+      <c r="H109" t="s">
+        <v>28</v>
+      </c>
+      <c r="I109" t="s">
+        <v>12</v>
+      </c>
+      <c r="J109">
+        <v>1000</v>
+      </c>
+      <c r="K109">
+        <v>1</v>
+      </c>
+      <c r="L109">
+        <v>1</v>
+      </c>
+      <c r="M109">
+        <v>0.5</v>
+      </c>
+      <c r="N109">
+        <v>1</v>
+      </c>
+      <c r="O109">
+        <v>15</v>
+      </c>
+      <c r="P109">
+        <v>1.5</v>
+      </c>
+      <c r="Q109">
+        <v>15.5</v>
+      </c>
+      <c r="S109">
+        <v>3</v>
+      </c>
+      <c r="T109">
+        <v>16.5</v>
+      </c>
+      <c r="W109">
+        <v>7</v>
+      </c>
+      <c r="X109">
+        <v>2</v>
+      </c>
+      <c r="Y109">
+        <v>2.5</v>
+      </c>
+      <c r="AA109">
+        <v>32.5</v>
+      </c>
+      <c r="AB109">
+        <v>3.5</v>
+      </c>
+      <c r="AC109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <v>33</v>
+      </c>
+      <c r="B110">
+        <v>2026</v>
+      </c>
+      <c r="C110">
+        <v>10</v>
+      </c>
+      <c r="D110">
+        <v>14</v>
+      </c>
+      <c r="E110">
+        <v>10</v>
+      </c>
+      <c r="F110">
+        <v>16</v>
+      </c>
+      <c r="G110" t="s">
+        <v>29</v>
+      </c>
+      <c r="H110" t="s">
+        <v>28</v>
+      </c>
+      <c r="I110" t="s">
+        <v>12</v>
+      </c>
+      <c r="J110">
+        <v>1000</v>
+      </c>
+      <c r="K110">
+        <v>1</v>
+      </c>
+      <c r="L110">
+        <v>1</v>
+      </c>
+      <c r="M110">
+        <v>0.5</v>
+      </c>
+      <c r="N110">
+        <v>1</v>
+      </c>
+      <c r="O110">
+        <v>16</v>
+      </c>
+      <c r="P110">
+        <v>2</v>
+      </c>
+      <c r="Q110">
+        <v>16.5</v>
+      </c>
+      <c r="S110">
+        <v>2.5</v>
+      </c>
+      <c r="U110">
+        <v>10.5</v>
+      </c>
+      <c r="W110">
+        <v>9.5</v>
+      </c>
+      <c r="X110">
+        <v>3</v>
+      </c>
+      <c r="Y110">
+        <v>2</v>
+      </c>
+      <c r="AA110">
+        <v>33.5</v>
+      </c>
+      <c r="AB110">
+        <v>3.5</v>
+      </c>
+      <c r="AC110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A111">
+        <v>34</v>
+      </c>
+      <c r="B111">
+        <v>2026</v>
+      </c>
+      <c r="C111">
+        <v>10</v>
+      </c>
+      <c r="D111">
+        <v>12</v>
+      </c>
+      <c r="E111">
+        <v>10</v>
+      </c>
+      <c r="F111">
+        <v>15</v>
+      </c>
+      <c r="G111" t="s">
+        <v>42</v>
+      </c>
+      <c r="H111" t="s">
+        <v>32</v>
+      </c>
+      <c r="I111" t="s">
+        <v>12</v>
+      </c>
+      <c r="J111">
+        <v>713</v>
+      </c>
+      <c r="K111">
+        <v>0</v>
+      </c>
+      <c r="L111">
+        <v>1</v>
+      </c>
+      <c r="M111">
+        <v>1</v>
+      </c>
+      <c r="N111" t="s">
+        <v>38</v>
+      </c>
+      <c r="O111">
+        <v>15</v>
+      </c>
+      <c r="P111">
+        <v>3</v>
+      </c>
+      <c r="Q111">
+        <v>14</v>
+      </c>
+      <c r="S111">
+        <v>6</v>
+      </c>
+      <c r="U111">
+        <v>10</v>
+      </c>
+      <c r="W111">
+        <v>9</v>
+      </c>
+      <c r="Y111">
+        <v>3</v>
+      </c>
+      <c r="AA111">
+        <v>37</v>
+      </c>
+      <c r="AB111">
+        <v>4</v>
+      </c>
+      <c r="AC111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <v>34</v>
+      </c>
+      <c r="B112">
+        <v>2026</v>
+      </c>
+      <c r="C112">
+        <v>10</v>
+      </c>
+      <c r="D112">
+        <v>12</v>
+      </c>
+      <c r="E112">
+        <v>10</v>
+      </c>
+      <c r="F112">
+        <v>15</v>
+      </c>
+      <c r="G112" t="s">
+        <v>42</v>
+      </c>
+      <c r="H112" t="s">
+        <v>32</v>
+      </c>
+      <c r="I112" t="s">
+        <v>12</v>
+      </c>
+      <c r="J112">
+        <v>721</v>
+      </c>
+      <c r="K112">
+        <v>0</v>
+      </c>
+      <c r="L112">
+        <v>1</v>
+      </c>
+      <c r="M112">
+        <v>1</v>
+      </c>
+      <c r="N112" t="s">
+        <v>38</v>
+      </c>
+      <c r="O112">
+        <v>15</v>
+      </c>
+      <c r="P112">
+        <v>3</v>
+      </c>
+      <c r="Q112">
+        <v>13</v>
+      </c>
+      <c r="S112">
+        <v>6</v>
+      </c>
+      <c r="T112">
+        <v>13</v>
+      </c>
+      <c r="U112">
+        <v>10</v>
+      </c>
+      <c r="W112">
+        <v>7</v>
+      </c>
+      <c r="Y112">
+        <v>3</v>
+      </c>
+      <c r="AA112">
+        <v>36</v>
+      </c>
+      <c r="AB112">
+        <v>3</v>
+      </c>
+      <c r="AC112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <v>34</v>
+      </c>
+      <c r="B113">
+        <v>2026</v>
+      </c>
+      <c r="C113">
+        <v>10</v>
+      </c>
+      <c r="D113">
+        <v>12</v>
+      </c>
+      <c r="E113">
+        <v>10</v>
+      </c>
+      <c r="F113">
+        <v>15</v>
+      </c>
+      <c r="G113" t="s">
+        <v>42</v>
+      </c>
+      <c r="H113" t="s">
+        <v>32</v>
+      </c>
+      <c r="I113" t="s">
+        <v>12</v>
+      </c>
+      <c r="J113">
+        <v>708</v>
+      </c>
+      <c r="K113">
+        <v>0</v>
+      </c>
+      <c r="L113">
+        <v>1</v>
+      </c>
+      <c r="M113">
+        <v>1</v>
+      </c>
+      <c r="N113">
+        <v>1</v>
+      </c>
+      <c r="O113">
+        <v>15</v>
+      </c>
+      <c r="P113">
+        <v>3</v>
+      </c>
+      <c r="R113">
+        <v>9</v>
+      </c>
+      <c r="S113">
+        <v>6</v>
+      </c>
+      <c r="T113">
+        <v>15</v>
+      </c>
+      <c r="W113">
+        <v>7</v>
+      </c>
+      <c r="Y113">
+        <v>3</v>
+      </c>
+      <c r="AA113">
+        <v>37</v>
+      </c>
+      <c r="AB113">
+        <v>4</v>
+      </c>
+      <c r="AC113">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update w/ ifop (10/19), harris (10/21), ipsos (10/22)
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3544FDE-0139-F94E-AC96-C927371347F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5E434F-1C5E-8A46-9416-56AD53301EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35620" yWindow="14060" windowWidth="28740" windowHeight="18800" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -567,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AC113"/>
+  <dimension ref="A1:AC120"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -8971,6 +8971,518 @@
         <v>0</v>
       </c>
     </row>
+    <row r="114" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>35</v>
+      </c>
+      <c r="B114">
+        <v>2026</v>
+      </c>
+      <c r="C114">
+        <v>10</v>
+      </c>
+      <c r="D114">
+        <v>17</v>
+      </c>
+      <c r="E114">
+        <v>10</v>
+      </c>
+      <c r="F114">
+        <v>19</v>
+      </c>
+      <c r="G114" t="s">
+        <v>11</v>
+      </c>
+      <c r="H114" t="s">
+        <v>13</v>
+      </c>
+      <c r="I114" t="s">
+        <v>12</v>
+      </c>
+      <c r="J114">
+        <v>1145</v>
+      </c>
+      <c r="K114">
+        <v>0</v>
+      </c>
+      <c r="L114">
+        <v>1</v>
+      </c>
+      <c r="M114">
+        <v>0.5</v>
+      </c>
+      <c r="N114">
+        <v>0.5</v>
+      </c>
+      <c r="O114">
+        <v>16.5</v>
+      </c>
+      <c r="P114">
+        <v>2.5</v>
+      </c>
+      <c r="Q114">
+        <v>14</v>
+      </c>
+      <c r="S114">
+        <v>3</v>
+      </c>
+      <c r="T114">
+        <v>15</v>
+      </c>
+      <c r="W114">
+        <v>7.5</v>
+      </c>
+      <c r="Y114">
+        <v>1.5</v>
+      </c>
+      <c r="AA114">
+        <v>36</v>
+      </c>
+      <c r="AB114">
+        <v>3.5</v>
+      </c>
+      <c r="AC114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>35</v>
+      </c>
+      <c r="B115">
+        <v>2026</v>
+      </c>
+      <c r="C115">
+        <v>10</v>
+      </c>
+      <c r="D115">
+        <v>17</v>
+      </c>
+      <c r="E115">
+        <v>10</v>
+      </c>
+      <c r="F115">
+        <v>19</v>
+      </c>
+      <c r="G115" t="s">
+        <v>11</v>
+      </c>
+      <c r="H115" t="s">
+        <v>13</v>
+      </c>
+      <c r="I115" t="s">
+        <v>12</v>
+      </c>
+      <c r="J115">
+        <v>1129</v>
+      </c>
+      <c r="K115">
+        <v>0</v>
+      </c>
+      <c r="L115">
+        <v>1</v>
+      </c>
+      <c r="M115">
+        <v>0.5</v>
+      </c>
+      <c r="N115">
+        <v>0.5</v>
+      </c>
+      <c r="O115">
+        <v>16</v>
+      </c>
+      <c r="P115">
+        <v>2</v>
+      </c>
+      <c r="Q115">
+        <v>16</v>
+      </c>
+      <c r="S115">
+        <v>3</v>
+      </c>
+      <c r="U115">
+        <v>13</v>
+      </c>
+      <c r="W115">
+        <v>7</v>
+      </c>
+      <c r="Y115">
+        <v>1.5</v>
+      </c>
+      <c r="AA115">
+        <v>38</v>
+      </c>
+      <c r="AB115">
+        <v>3</v>
+      </c>
+      <c r="AC115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>35</v>
+      </c>
+      <c r="B116">
+        <v>2026</v>
+      </c>
+      <c r="C116">
+        <v>10</v>
+      </c>
+      <c r="D116">
+        <v>17</v>
+      </c>
+      <c r="E116">
+        <v>10</v>
+      </c>
+      <c r="F116">
+        <v>19</v>
+      </c>
+      <c r="G116" t="s">
+        <v>11</v>
+      </c>
+      <c r="H116" t="s">
+        <v>13</v>
+      </c>
+      <c r="I116" t="s">
+        <v>12</v>
+      </c>
+      <c r="J116">
+        <v>1138</v>
+      </c>
+      <c r="K116">
+        <v>0</v>
+      </c>
+      <c r="L116">
+        <v>1</v>
+      </c>
+      <c r="M116">
+        <v>0.5</v>
+      </c>
+      <c r="N116">
+        <v>0.5</v>
+      </c>
+      <c r="O116">
+        <v>18</v>
+      </c>
+      <c r="Q116">
+        <v>16</v>
+      </c>
+      <c r="T116">
+        <v>16</v>
+      </c>
+      <c r="W116">
+        <v>6.5</v>
+      </c>
+      <c r="Y116">
+        <v>2.5</v>
+      </c>
+      <c r="AA116">
+        <v>37</v>
+      </c>
+      <c r="AB116">
+        <v>3.5</v>
+      </c>
+      <c r="AC116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <v>36</v>
+      </c>
+      <c r="B117">
+        <v>2026</v>
+      </c>
+      <c r="C117">
+        <v>10</v>
+      </c>
+      <c r="D117">
+        <v>19</v>
+      </c>
+      <c r="E117">
+        <v>10</v>
+      </c>
+      <c r="F117">
+        <v>21</v>
+      </c>
+      <c r="G117" t="s">
+        <v>31</v>
+      </c>
+      <c r="H117" t="s">
+        <v>32</v>
+      </c>
+      <c r="I117" t="s">
+        <v>12</v>
+      </c>
+      <c r="J117">
+        <v>1759</v>
+      </c>
+      <c r="K117">
+        <v>0</v>
+      </c>
+      <c r="L117">
+        <v>1</v>
+      </c>
+      <c r="M117">
+        <v>1</v>
+      </c>
+      <c r="N117">
+        <v>1</v>
+      </c>
+      <c r="O117">
+        <v>17</v>
+      </c>
+      <c r="P117">
+        <v>2</v>
+      </c>
+      <c r="Q117">
+        <v>13</v>
+      </c>
+      <c r="S117">
+        <v>2</v>
+      </c>
+      <c r="T117">
+        <v>16</v>
+      </c>
+      <c r="W117">
+        <v>7</v>
+      </c>
+      <c r="Y117">
+        <v>2</v>
+      </c>
+      <c r="AA117">
+        <v>35</v>
+      </c>
+      <c r="AB117">
+        <v>5</v>
+      </c>
+      <c r="AC117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <v>36</v>
+      </c>
+      <c r="B118">
+        <v>2026</v>
+      </c>
+      <c r="C118">
+        <v>10</v>
+      </c>
+      <c r="D118">
+        <v>19</v>
+      </c>
+      <c r="E118">
+        <v>10</v>
+      </c>
+      <c r="F118">
+        <v>21</v>
+      </c>
+      <c r="G118" t="s">
+        <v>31</v>
+      </c>
+      <c r="H118" t="s">
+        <v>32</v>
+      </c>
+      <c r="I118" t="s">
+        <v>12</v>
+      </c>
+      <c r="J118">
+        <v>1717</v>
+      </c>
+      <c r="K118">
+        <v>0</v>
+      </c>
+      <c r="L118">
+        <v>1</v>
+      </c>
+      <c r="M118">
+        <v>1</v>
+      </c>
+      <c r="N118">
+        <v>1</v>
+      </c>
+      <c r="O118">
+        <v>19</v>
+      </c>
+      <c r="P118">
+        <v>2</v>
+      </c>
+      <c r="Q118">
+        <v>13</v>
+      </c>
+      <c r="S118">
+        <v>2</v>
+      </c>
+      <c r="U118">
+        <v>11</v>
+      </c>
+      <c r="W118">
+        <v>9</v>
+      </c>
+      <c r="Y118">
+        <v>2</v>
+      </c>
+      <c r="AA118">
+        <v>35</v>
+      </c>
+      <c r="AB118">
+        <v>6</v>
+      </c>
+      <c r="AC118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <v>37</v>
+      </c>
+      <c r="B119">
+        <v>2026</v>
+      </c>
+      <c r="C119">
+        <v>10</v>
+      </c>
+      <c r="D119">
+        <v>21</v>
+      </c>
+      <c r="E119">
+        <v>10</v>
+      </c>
+      <c r="F119">
+        <v>22</v>
+      </c>
+      <c r="G119" t="s">
+        <v>33</v>
+      </c>
+      <c r="H119" t="s">
+        <v>13</v>
+      </c>
+      <c r="I119" t="s">
+        <v>12</v>
+      </c>
+      <c r="J119">
+        <v>1060</v>
+      </c>
+      <c r="K119">
+        <v>0</v>
+      </c>
+      <c r="L119">
+        <v>1</v>
+      </c>
+      <c r="M119">
+        <v>0.5</v>
+      </c>
+      <c r="N119">
+        <v>0.5</v>
+      </c>
+      <c r="O119">
+        <v>17</v>
+      </c>
+      <c r="P119">
+        <v>2</v>
+      </c>
+      <c r="Q119">
+        <v>14</v>
+      </c>
+      <c r="S119">
+        <v>3.5</v>
+      </c>
+      <c r="T119">
+        <v>15</v>
+      </c>
+      <c r="W119">
+        <v>8</v>
+      </c>
+      <c r="Y119">
+        <v>2</v>
+      </c>
+      <c r="AA119">
+        <v>33.5</v>
+      </c>
+      <c r="AB119">
+        <v>4.5</v>
+      </c>
+      <c r="AC119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <v>37</v>
+      </c>
+      <c r="B120">
+        <v>2026</v>
+      </c>
+      <c r="C120">
+        <v>10</v>
+      </c>
+      <c r="D120">
+        <v>21</v>
+      </c>
+      <c r="E120">
+        <v>10</v>
+      </c>
+      <c r="F120">
+        <v>22</v>
+      </c>
+      <c r="G120" t="s">
+        <v>33</v>
+      </c>
+      <c r="H120" t="s">
+        <v>13</v>
+      </c>
+      <c r="I120" t="s">
+        <v>12</v>
+      </c>
+      <c r="J120">
+        <v>1048</v>
+      </c>
+      <c r="K120">
+        <v>0</v>
+      </c>
+      <c r="L120">
+        <v>1</v>
+      </c>
+      <c r="M120">
+        <v>0.5</v>
+      </c>
+      <c r="N120">
+        <v>0.5</v>
+      </c>
+      <c r="O120">
+        <v>17</v>
+      </c>
+      <c r="P120">
+        <v>2.5</v>
+      </c>
+      <c r="Q120">
+        <v>15.5</v>
+      </c>
+      <c r="S120">
+        <v>3.5</v>
+      </c>
+      <c r="U120">
+        <v>9.5</v>
+      </c>
+      <c r="W120">
+        <v>11.5</v>
+      </c>
+      <c r="Y120">
+        <v>2</v>
+      </c>
+      <c r="AA120">
+        <v>33.5</v>
+      </c>
+      <c r="AB120">
+        <v>4.5</v>
+      </c>
+      <c r="AC120">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update w/ cluster17 (10/22)
</commit_message>
<xml_diff>
--- a/polls_data_2027.xlsx
+++ b/polls_data_2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/flavienganter/Documents/Polls Présidentielle 2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5E434F-1C5E-8A46-9416-56AD53301EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BCD96E-7C71-B34C-AA22-18BCC1569840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
+    <workbookView xWindow="38400" yWindow="-760" windowWidth="30240" windowHeight="18980" xr2:uid="{090D314A-8FCB-D940-B611-DA3362EC34C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -567,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4382087-D1FD-6B45-998E-95CA20172B84}">
-  <dimension ref="A1:AC120"/>
+  <dimension ref="A1:AC122"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
@@ -9483,6 +9483,154 @@
         <v>0</v>
       </c>
     </row>
+    <row r="121" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>38</v>
+      </c>
+      <c r="B121">
+        <v>2026</v>
+      </c>
+      <c r="C121">
+        <v>10</v>
+      </c>
+      <c r="D121">
+        <v>19</v>
+      </c>
+      <c r="E121">
+        <v>10</v>
+      </c>
+      <c r="F121">
+        <v>22</v>
+      </c>
+      <c r="G121" t="s">
+        <v>40</v>
+      </c>
+      <c r="H121" t="s">
+        <v>32</v>
+      </c>
+      <c r="I121" t="s">
+        <v>12</v>
+      </c>
+      <c r="J121">
+        <v>1920</v>
+      </c>
+      <c r="K121">
+        <v>0</v>
+      </c>
+      <c r="L121">
+        <v>1</v>
+      </c>
+      <c r="M121">
+        <v>0.1</v>
+      </c>
+      <c r="N121">
+        <v>0.4</v>
+      </c>
+      <c r="O121">
+        <v>18.5</v>
+      </c>
+      <c r="P121">
+        <v>2</v>
+      </c>
+      <c r="Q121">
+        <v>13.1</v>
+      </c>
+      <c r="S121">
+        <v>2</v>
+      </c>
+      <c r="T121">
+        <v>16</v>
+      </c>
+      <c r="W121">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="Y121">
+        <v>3</v>
+      </c>
+      <c r="AA121">
+        <v>32.9</v>
+      </c>
+      <c r="AB121">
+        <v>3.8</v>
+      </c>
+      <c r="AC121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>38</v>
+      </c>
+      <c r="B122">
+        <v>2026</v>
+      </c>
+      <c r="C122">
+        <v>10</v>
+      </c>
+      <c r="D122">
+        <v>19</v>
+      </c>
+      <c r="E122">
+        <v>10</v>
+      </c>
+      <c r="F122">
+        <v>22</v>
+      </c>
+      <c r="G122" t="s">
+        <v>40</v>
+      </c>
+      <c r="H122" t="s">
+        <v>32</v>
+      </c>
+      <c r="I122" t="s">
+        <v>12</v>
+      </c>
+      <c r="J122">
+        <v>1889</v>
+      </c>
+      <c r="K122">
+        <v>0</v>
+      </c>
+      <c r="L122">
+        <v>1</v>
+      </c>
+      <c r="M122">
+        <v>0.1</v>
+      </c>
+      <c r="N122">
+        <v>0.4</v>
+      </c>
+      <c r="O122">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="P122">
+        <v>2</v>
+      </c>
+      <c r="Q122">
+        <v>14.2</v>
+      </c>
+      <c r="S122">
+        <v>1.8</v>
+      </c>
+      <c r="U122">
+        <v>11.9</v>
+      </c>
+      <c r="W122">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="Y122">
+        <v>3.5</v>
+      </c>
+      <c r="AA122">
+        <v>32.5</v>
+      </c>
+      <c r="AB122">
+        <v>3.9</v>
+      </c>
+      <c r="AC122">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>